<commit_message>
Fill Claude reviews for new CPE-expansion rows; drop stale disagreement/mining files
- Judge all 2,120 blank Claude review rows across categories (streaming,
  cameras, alarms, garden, smartspeakers, smartplugs, doorlock, babymonitor,
  hub, lighting, robotvacuum) against the per-category scope notes.
- Remove regenerable/settled intermediates: human_disagreements.csv,
  human_disagreement_resolutions.csv, RECALL_MINING_SUMMARY.md.
</commit_message>
<xml_diff>
--- a/data/vendor-search/results_all_airconditioner.xlsx
+++ b/data/vendor-search/results_all_airconditioner.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I125"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,12 +454,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Lizzie Judgment</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Cukier Judgment</t>
+          <t>matched_terms</t>
         </is>
       </c>
     </row>
@@ -482,8 +477,10 @@
       <c r="D2" t="n">
         <v>5</v>
       </c>
-      <c r="E2" t="n">
-        <v>2</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
@@ -493,12 +490,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>fujitsu</t>
         </is>
       </c>
     </row>
@@ -521,8 +513,10 @@
       <c r="D3" t="n">
         <v>7.2</v>
       </c>
-      <c r="E3" t="n">
-        <v>2</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -534,8 +528,11 @@
           <t>cpe:2.3:a:fujitsu:siemens_networker:6.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -556,8 +553,10 @@
       <c r="D4" t="n">
         <v>5</v>
       </c>
-      <c r="E4" t="n">
-        <v>2</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
@@ -565,8 +564,11 @@
           <t>cpe:2.3:h:fujitsu:netshelter_fw:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:netshelter_fw-l:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:netshelter_fw-m:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:netshelter_fw-p:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -587,8 +589,10 @@
       <c r="D5" t="n">
         <v>7.5</v>
       </c>
-      <c r="E5" t="n">
-        <v>2</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
@@ -596,8 +600,11 @@
           <t>cpe:2.3:a:fujitsu:myweb_portal_office:*:*:citizen:*:*:*:*:*|cpe:2.3:a:fujitsu:myweb_portal_office:*:*:light:*:*:*:*:*|cpe:2.3:a:fujitsu:myweb_portal_office:*:*:medical:*:*:*:*:*|cpe:2.3:a:fujitsu:myweb_portal_office:*:*:public:*:*:*:*:*|cpe:2.3:a:fujitsu:myweb_portal_office:*:*:school:*:*:*:*:*|cpe:2.3:a:fujitsu:myweb_portal_office:*:*:standard:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -618,8 +625,10 @@
       <c r="D6" t="n">
         <v>4.6</v>
       </c>
-      <c r="E6" t="n">
-        <v>2</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
@@ -627,8 +636,11 @@
           <t>cpe:2.3:a:jochen_friedrich:pinball:0.3.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>friedrich</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -649,8 +661,10 @@
       <c r="D7" t="n">
         <v>5</v>
       </c>
-      <c r="E7" t="n">
-        <v>2</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
@@ -658,8 +672,11 @@
           <t>cpe:2.3:a:fujitsu:serverview:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:2.50:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -680,8 +697,10 @@
       <c r="D8" t="n">
         <v>4.3</v>
       </c>
-      <c r="E8" t="n">
-        <v>2</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -693,8 +712,11 @@
           <t>cpe:2.3:a:fujitsu:serverview:2.50:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:3.60l98:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.10l11:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.10l81:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -715,8 +737,10 @@
       <c r="D9" t="n">
         <v>10</v>
       </c>
-      <c r="E9" t="n">
-        <v>2</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -728,8 +752,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.0:*:rehl_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.0:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.0:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.0:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.1:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.2:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.2:*:rhel_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.2:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.2:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.3:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.3:*:rhel_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.3:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.3:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:rhel_as4_ipf:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:rhel_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:rhel5_intel64:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:rhel5_ipf:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:rhel5_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0a:*:rhel_as4_ipf:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0a:*:rhel5_ipf:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0a:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.0:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.0:*:rhel_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.0:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.0:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.2:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.2:*:rhel_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.2:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.2:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.3:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.3:*:rhel_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.3:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.3:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:rhel_as4_em64t:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:rhel_as4_ipf:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:rhel_as4_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:rhel5_intel64:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:rhel5_ipf:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:rhel5_x86:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:solaris:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0.0:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0a:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_enterprise:8.0.0:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_standard_j:8.0.0:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_enterprise:8.0.1:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_enterprise:v9.0.0:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_standard_j:8.0.1:*:windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_standard_j:v9.0.0:*:windows:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -750,8 +777,10 @@
       <c r="D10" t="n">
         <v>5</v>
       </c>
-      <c r="E10" t="n">
-        <v>2</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -763,8 +792,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server_enterprise:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:7.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:7.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_enterprise:8.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_modelers_j:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_standard_j:8.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_business_application_server:8.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_smart_repository:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -785,8 +817,10 @@
       <c r="D11" t="n">
         <v>6.4</v>
       </c>
-      <c r="E11" t="n">
-        <v>2</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
@@ -794,8 +828,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server:3.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:3.0:*:standard:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.0:*:standard:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.0:*:web_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.1:*:standard:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.1:*:web_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:standard:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:web_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0.1:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0.1:*:plus_developer:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:6.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:6.0:*:plus:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:standard:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:plus:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -816,8 +853,10 @@
       <c r="D12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="n">
-        <v>2</v>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -829,8 +868,11 @@
           <t>cpe:2.3:a:fujitsu:e-pares:l01:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l03:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l10:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l20:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l30:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:v01:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -851,8 +893,10 @@
       <c r="D13" t="n">
         <v>4.3</v>
       </c>
-      <c r="E13" t="n">
-        <v>2</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -864,8 +908,11 @@
           <t>cpe:2.3:a:fujitsu:e-pares:l01:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:v01:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -886,8 +933,10 @@
       <c r="D14" t="n">
         <v>2.6</v>
       </c>
-      <c r="E14" t="n">
-        <v>2</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -899,8 +948,11 @@
           <t>cpe:2.3:a:fujitsu:e-pares:l01:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l03:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l10:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l20:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l30:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:l40:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:e-pares:v01:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -921,8 +973,10 @@
       <c r="D15" t="n">
         <v>4.6</v>
       </c>
-      <c r="E15" t="n">
-        <v>2</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
@@ -930,8 +984,11 @@
           <t>cpe:2.3:o:disney_interactive:disney_mobile:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:f-08d:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:arrows_tab_lte_f-01d:*:*:*:*:*:*:*:*|cpe:2.3:h:sharp:softbank_102sh:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:regza_phone_t-01d:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:arrows_x_lte_f-05d:-:*:*:*:*:*:*:*|cpe:2.3:h:lg:prada_phone_l-02d:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -952,8 +1009,10 @@
       <c r="D16" t="n">
         <v>7.2</v>
       </c>
-      <c r="E16" t="n">
-        <v>2</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -965,8 +1024,11 @@
           <t>cpe:2.3:h:fujitsu:arrows_kiss_f-03d:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:arrows_tab_lte_f-01d:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:f-12c:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:regza_phone_t-01d:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -987,8 +1049,10 @@
       <c r="D17" t="n">
         <v>4.6</v>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
@@ -996,8 +1060,11 @@
           <t>cpe:2.3:h:fujitsu:arrows_me_f-11d:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1018,8 +1085,10 @@
       <c r="D18" t="n">
         <v>8.1</v>
       </c>
-      <c r="E18" t="n">
-        <v>3</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1031,8 +1100,11 @@
           <t>cpe:2.3:o:debian:debian_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:12.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:14.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:15.10:*:*:*:*:*:*:*|cpe:2.3:a:hp:helion_openstack:1.1.1:*:*:*:*:*:*:*|cpe:2.3:a:hp:helion_openstack:2.0.0:*:*:*:*:*:*:*|cpe:2.3:a:hp:helion_openstack:2.1.0:*:*:*:*:*:*:*|cpe:2.3:a:hp:server_migration_pack:7.5:*:*:*:*:*:*:*|cpe:2.3:a:sophos:unified_threat_management_software:9.319:*:*:*:*:*:*:*|cpe:2.3:a:sophos:unified_threat_management_software:9.355:*:*:*:*:*:*:*|cpe:2.3:a:suse:linux_enterprise_debuginfo:11.0:sp2:*:*:*:*:*:*|cpe:2.3:a:suse:linux_enterprise_debuginfo:11.0:sp3:*:*:*:*:*:*|cpe:2.3:a:suse:linux_enterprise_debuginfo:11.0:sp4:*:*:*:*:*:*|cpe:2.3:o:opensuse:opensuse:13.2:*:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_desktop:11.0:sp3:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_desktop:11.0:sp4:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_desktop:12:*:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_desktop:12:sp1:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:11.0:sp2:*:*:lts:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:11.0:sp3:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:11.0:sp3:*:*:*:vmware:*:*|cpe:2.3:o:suse:linux_enterprise_server:11.0:sp4:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:12:sp1:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_software_development_kit:11.0:sp3:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_software_development_kit:11.0:sp4:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_software_development_kit:12:*:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_software_development_kit:12:sp1:*:*:*:*:*:*|cpe:2.3:o:suse:suse_linux_enterprise_server:12:*:*:*:*:*:*:*|cpe:2.3:a:oracle:exalogic_infrastructure:1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:exalogic_infrastructure:2.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_access_policy_manager:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_advanced_firewall_manager:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_analytics:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_application_acceleration_manager:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_application_security_manager:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_domain_name_system:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_link_controller:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_local_traffic_manager:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:f5:big-ip_policy_enforcement_manager:12.0.0:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m10_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_desktop:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_hpc_node:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_hpc_node_eus:7.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_eus:7.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_workstation:7.0:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.9:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.10:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.10.1:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.11:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.11.1:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.11.2:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.11.3:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.12:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.12.1:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.12.2:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.13:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.14:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.14.1:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.15:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.16:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.17:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.18:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.19:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.20:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.21:*:*:*:*:*:*:*|cpe:2.3:a:gnu:glibc:2.22:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1053,8 +1125,10 @@
       <c r="D19" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E19" t="n">
-        <v>3</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1066,8 +1140,11 @@
           <t>cpe:2.3:o:trane:comfortlink_ii_firmware:2.0.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>trane comfortlink</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1088,8 +1165,10 @@
       <c r="D20" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E20" t="n">
-        <v>3</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1101,8 +1180,11 @@
           <t>cpe:2.3:o:trane:comfortlink_ii_firmware:2.0.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>trane comfortlink</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1123,8 +1205,10 @@
       <c r="D21" t="n">
         <v>7.8</v>
       </c>
-      <c r="E21" t="n">
-        <v>3</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1136,8 +1220,11 @@
           <t>cpe:2.3:a:fujitsu:fence-explorer:*:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_10:-:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_7:-:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_8.1:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1158,8 +1245,10 @@
       <c r="D22" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E22" t="n">
-        <v>3.1</v>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1167,8 +1256,11 @@
           <t>cpe:2.3:a:haxx:curl:*:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:7.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:9.0:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:12.04:*:*:*:esm:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:14.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:16.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:17.10:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_desktop:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_eus:7.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_eus:7.5:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_workstation:7.0:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1189,8 +1281,10 @@
       <c r="D23" t="n">
         <v>5.6</v>
       </c>
-      <c r="E23" t="n">
-        <v>3.1</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
@@ -1198,8 +1292,11 @@
           <t>cpe:2.3:h:intel:atom_c:c2308:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2316:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2338:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2350:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2358:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2508:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2516:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2518:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2530:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2538:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2550:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2558:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2718:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2730:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2738:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2750:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c2758:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3308:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3338:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3508:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3538:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3558:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3708:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3750:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3758:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3808:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3830:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3850:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3858:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3950:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3955:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_c:c3958:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_e:e3805:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_e:e3815:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_e:e3825:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_e:e3826:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_e:e3827:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_e:e3845:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3130:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3200rk:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3205rk:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3230rk:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3235rk:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3265rk:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3295rk:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3405:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_x3:c3445:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z2420:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z2460:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z2480:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z2520:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z2560:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z2580:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z2760:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3460:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3480:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3530:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3560:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3570:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3580:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3590:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3735d:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3735e:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3735f:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3735g:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3736f:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3736g:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3740:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3740d:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3745:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3745d:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3770:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3770d:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3775:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3775d:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3785:*:*:*:*:*:*:*|cpe:2.3:h:intel:atom_z:z3795:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j1750:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j1800:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j1850:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j1900:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j3060:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j3160:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j3355:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j3455:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j4005:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_j:j4105:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2805:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2806:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2807:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2808:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2810:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2815:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2820:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2830:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2840:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2910:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2920:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2930:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n2940:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3000:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3010:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3050:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3060:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3150:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3160:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3350:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n3450:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n4000:*:*:*:*:*:*:*|cpe:2.3:h:intel:celeron_n:n4100:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:330e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:330m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:330um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:350m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:370m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:380m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:380um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:390m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:530:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:540:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:550:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:560:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2100:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2100t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2102:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2105:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2115c:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2120:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2120t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2125:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2130:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2310e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2310m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2312m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2328m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2330e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2330m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2340ue:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2348m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2350m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2357m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2365m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2367m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2370m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2375m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:2377m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3110m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3115c:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3120m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3120me:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3130m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3210:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3217u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3217ue:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3220:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3220t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3225:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3227u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3229y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3240:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3240t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3245:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3250:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:3250t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4000m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4005u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4010u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4010y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4012y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4020y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4025u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4030u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4030y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4100e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4100m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4100u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4102e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4110e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4110m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4112e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4120u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4130:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4130t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4150:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4150t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4158u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4160:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4160t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4170:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4170t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4330:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4330t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4330te:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4340:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4340te:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4350:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4350t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4360:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4360t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4370:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:4370t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:5005u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:5010u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:5015u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:5020u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:5157u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6006u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6098p:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6100:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6100e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6100h:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6100t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6100te:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6100u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6102e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6157u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6167u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6300:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6300t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:6320:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:8100:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i3:8350k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:430m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:430um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:450m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:460m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:470um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:480m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:520e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:520m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:520um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:540m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:540um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:560m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:560um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:580m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:650:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:655k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:660:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:661:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:670:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:680:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:750:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:750s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:760:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2300:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2310:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2320:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2380p:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2390t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2400:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2400s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2405s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2410m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2430m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2435m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2450m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2450p:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2467m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2500:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2500k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2500s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2500t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2510e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2515e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2520m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2537m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2540m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2550k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:2557m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3210m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3230m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3317u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3320m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3330:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3330s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3337u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3339y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3340:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3340m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3340s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3350p:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3360m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3380m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3427u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3437u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3439y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3450:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3450s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3470:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3470s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3470t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3475s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3550:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3550s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3570:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3570k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3570s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3570t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:3610me:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4200h:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4200m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4200u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4200y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4202y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4210h:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4210m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4210u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4210y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4220y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4250u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4258u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4260u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4278u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4288u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4300m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4300u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4300y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4302y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4308u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4310m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4310u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4330m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4340m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4350u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4360u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4400e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4402e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4402ec:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4410e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4422e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4430:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4430s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4440:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4440s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4460:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4460s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4460t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4570:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4570r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4570s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4570t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4570te:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4590:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4590s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4590t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4670:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4670k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4670r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4670s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4670t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4690:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4690k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4690s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:4690t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5200u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5250u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5257u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5287u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5300u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5350h:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5350u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5575r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5675c:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:5675r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6200u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6260u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6267u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6287u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6300hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6300u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6350hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6360u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6400:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6400t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6402p:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6440eq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6440hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6442eq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6500:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6500t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6500te:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6585r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6600:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6600k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6600t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:6685r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:8250u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:8350u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:8400:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i5:8600k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7y75:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:610e:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:620le:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:620lm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:620m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:620ue:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:620um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:640lm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:640m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:640um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:660lm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:660ue:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:660um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:680um:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:720qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:740qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:820qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:840qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:860:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:860s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:870:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:870s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:875k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:880:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:920:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:920xm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:930:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:940:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:940xm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:950:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:960:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:965:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:970:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:975:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:980:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:980x:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:990x:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2600:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2600k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2600s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2610ue:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2617m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2620m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2629m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2630qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2635qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2637m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2640m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2649m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2655le:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2657m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2670qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2675qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2677m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2700k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2710qe:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2715qe:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2720qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2760qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2820qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2860qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2920xm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:2960xm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3517u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3517ue:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3520m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3537u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3540m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3555le:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3610qe:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3610qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3612qe:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3612qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3615qe:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3615qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3630qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3632qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3635qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3667u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3687u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3689y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3720qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3740qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3770:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3770k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3770s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3770t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3820qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:3840qm:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4500u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4510u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4550u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4558u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4578u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4600m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4600u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4610m:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4610y:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4650u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4700ec:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4700eq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4700hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4700mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4702ec:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4702hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4702mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4710hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4710mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4712hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4712mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4720hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4722hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4750hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4760hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4765t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4770:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4770hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4770k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4770r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4770s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4770t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4770te:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4771:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4785t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4790:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4790k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4790s:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4790t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4800mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4810mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4850hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4860hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4870hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4900mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4910mq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4950hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4960hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:4980hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5500u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5550u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5557u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5600u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5650u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5700eq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5700hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5750hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5775c:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5775r:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5850eq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5850hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:5950hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7500u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7560u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7567u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7600u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7660u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7700:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7700hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7700k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7700t:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7820eq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7820hk:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7820hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:7920hq:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:8550u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:8650u:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:8700:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_i7:8700k:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m:5y10:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m:5y10a:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m:5y10c:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m:5y31:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m:5y51:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m:5y70:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m:5y71:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m3:6y30:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m3:7y30:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m3:7y32:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m5:6y54:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m5:6y57:*:*:*:*:*:*:*|cpe:2.3:h:intel:core_m7:6y75:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_j:j2850:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_j:j2900:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_j:j3710:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_j:j4205:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_n:n3510:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_n:n3520:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_n:n3530:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_n:n3540:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_n:n3700:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_n:n3710:*:*:*:*:*:*:*|cpe:2.3:h:intel:pentium_n:n4200:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5502:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5503:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5504:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5506:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5507:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5520:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5530:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5540:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5603:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5606:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5607:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5620:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5630:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5640:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5645:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e5649:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e6510:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e6540:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e7520:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e7530:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:e7540:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:ec5509:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:ec5539:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:ec5549:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l3406:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l3426:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5506:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5508:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5518:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5520:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5530:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5609:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5618:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5630:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5638:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l5640:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l7545:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:l7555:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:lc5518:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:lc5528:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:w3670:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:w3680:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:w3690:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:w5580:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:w5590:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x3430:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x3440:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x3450:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x3460:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x3470:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x3480:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5550:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5560:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5570:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5647:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5650:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5660:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5667:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5670:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5672:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5675:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5677:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5680:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5687:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x5690:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x6550:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x7542:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x7550:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon:x7560:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_bronze_3104:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_bronze_3106:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e-1105c:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1505m_v6:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1515m_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1535m_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1535m_v6:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1545m_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1558l_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1565l_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1575m_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1578l_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1585_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3:1585l_v5:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1105c_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1125c:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1125c_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1220:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1220_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1220_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1220_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1220_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_12201:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_12201_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1220l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1225:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1225_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1225_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1225_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1225_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1226_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1230:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1230_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1230_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1230_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1230_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1230l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1231_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1235:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1235l_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1240:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1240_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1240_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1240_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1240_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1240l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1240l_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1241_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1245:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1245_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1245_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1245_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1245_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1246_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1258l_v4:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1260l:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1260l_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1265l_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1265l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1265l_v4:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1268l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1268l_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1270:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1270_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1270_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1270_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1270_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1271_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1275:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1275_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1275_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1275_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1275_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1275l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1276_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1278l_v4:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1280:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1280_v2:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1280_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1280_v5:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1280_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1281_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1285_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1285_v4:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1285_v6:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1285l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1285l_v4:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1286_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1286l_v3:-:*:*:*:*:*:*:*|cpe:2.3:h:intel:xeon_e3_1290:-:*:*:*:*:*:*:*|cpe:2.3:h:</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1220,8 +1317,10 @@
       <c r="D24" t="n">
         <v>6.8</v>
       </c>
-      <c r="E24" t="n">
-        <v>3.1</v>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1233,8 +1332,11 @@
           <t>cpe:2.3:a:openbsd:openssh:*:*:*:*:*:*:*:*|cpe:2.3:a:winscp:winscp:*:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:14.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:16.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.10:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:9.0:*:*:*:*:*:*:*|cpe:2.3:a:netapp:element_software:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:ontap_select_deploy:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:storage_automation_store:-:*:*:*:*:*:*:*|cpe:2.3:o:fedoraproject:fedora:30:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.1:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:siemens:scalance_x204rna_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:siemens:scalance_x204rna:-:*:*:*:*:*:*:*|cpe:2.3:o:siemens:scalance_x204rna_eec_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:siemens:scalance_x204rna_eec:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1255,8 +1357,10 @@
       <c r="D25" t="n">
         <v>5.9</v>
       </c>
-      <c r="E25" t="n">
-        <v>3.1</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1268,8 +1372,11 @@
           <t>cpe:2.3:a:openbsd:openssh:*:*:*:*:*:*:*:*|cpe:2.3:a:winscp:winscp:*:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:14.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:16.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.10:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:9.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.1:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:fedoraproject:fedora:30:*:*:*:*:*:*:*|cpe:2.3:a:apache:mina_sshd:2.2.0:*:*:*:*:*:*:*|cpe:2.3:o:freebsd:freebsd:*:*:*:*:*:*:*:*|cpe:2.3:o:freebsd:freebsd:12.0:-:*:*:*:*:*:*|cpe:2.3:o:freebsd:freebsd:12.0:p1:*:*:*:*:*:*|cpe:2.3:o:freebsd:freebsd:12.0:p2:*:*:*:*:*:*|cpe:2.3:o:freebsd:freebsd:12.0:p3:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:o:siemens:scalance_x204rna_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:siemens:scalance_x204rna:-:*:*:*:*:*:*:*|cpe:2.3:o:siemens:scalance_x204rna_eec_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:siemens:scalance_x204rna_eec:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1290,8 +1397,10 @@
       <c r="D26" t="n">
         <v>4.2</v>
       </c>
-      <c r="E26" t="n">
-        <v>3.1</v>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -1299,8 +1408,11 @@
           <t>cpe:2.3:o:mi:mi_5s_plus_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:mi:mi_5s_plus:-:*:*:*:*:*:*:*|cpe:2.3:o:sony:xperia_z4_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:sony:xperia_z4:-:*:*:*:*:*:*:*|cpe:2.3:o:samsung:galaxy_s6_edge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:samsung:galaxy_s6_edge:-:*:*:*:*:*:*:*|cpe:2.3:o:samsung:galaxy_s4_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:samsung:galaxy_s4:-:*:*:*:*:*:*:*|cpe:2.3:o:google:nexus_7_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:google:nexus_7:-:*:*:*:*:*:*:*|cpe:2.3:o:google:nexus_9_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:google:nexus_9:-:*:*:*:*:*:*:*|cpe:2.3:o:sharp:aquos_zeta_sh-04f_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:sharp:aquos_zeta_sh-04f:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:arrows_nx_f05-f_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:arrows_nx_f05-f:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1321,8 +1433,10 @@
       <c r="D27" t="n">
         <v>6.1</v>
       </c>
-      <c r="E27" t="n">
-        <v>3.1</v>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1334,8 +1448,11 @@
           <t>cpe:2.3:a:redhat:hibernate_validator:*:*:*:*:*:*:*:*|cpe:2.3:a:redhat:hibernate_validator:6.1.0:alpha1:*:*:*:*:*:*|cpe:2.3:a:redhat:hibernate_validator:6.1.0:alpha2:*:*:*:*:*:*|cpe:2.3:a:redhat:hibernate_validator:6.1.0:alpha3:*:*:*:*:*:*|cpe:2.3:a:redhat:hibernate_validator:6.1.0:alpha4:*:*:*:*:*:*|cpe:2.3:a:redhat:hibernate_validator:6.1.0:alpha5:*:*:*:*:*:*|cpe:2.3:a:redhat:hibernate_validator:6.1.0:alpha6:*:*:*:*:*:*|cpe:2.3:a:redhat:fuse:1.0:*:*:*:*:*:*:*|cpe:2.3:a:redhat:jboss_data_grid:-:*:*:*:text-only:*:*:*|cpe:2.3:a:redhat:jboss_enterprise_application_platform:-:*:*:*:text-only:*:*:*|cpe:2.3:a:redhat:openshift_application_runtimes:-:*:*:*:text-only:*:*:*|cpe:2.3:a:redhat:single_sign-on:-:*:*:*:text-only:*:*:*|cpe:2.3:a:redhat:jboss_enterprise_application_platform:7.2:*:*:*:*:*:*:*|cpe:2.3:a:redhat:jboss_enterprise_application_platform:7.3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:6.0:*:*:*:*:*:*:*|cpe:2.3:a:netapp:active_iq_unified_manager:-:*:*:*:*:linux:*:*|cpe:2.3:a:netapp:active_iq_unified_manager:-:*:*:*:*:vmware_vsphere:*:*|cpe:2.3:a:netapp:active_iq_unified_manager:-:*:*:*:*:windows:*:*|cpe:2.3:a:netapp:management_services_for_element_software_and_netapp_hci:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:snapcenter_plug-in:-:*:*:*:*:vmware_vsphere:*:*|cpe:2.3:o:netapp:element:-:*:*:*:*:vcenter_server:*:*|cpe:2.3:a:oracle:access_manager:11.1.2.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:access_manager:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:access_manager:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:agile_engineering_data_management:6.2.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:agile_plm:9.3.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:agile_plm:9.3.6:*:*:*:*:*:*:*|cpe:2.3:a:oracle:agile_product_lifecycle_analytics:3.6.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:agile_product_lifecycle_management_integration_pack:3.6:*:*:*:*:e-business_suite:*:*|cpe:2.3:a:oracle:airlines_data_model:12.1.1.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:airlines_data_model:12.2.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:application_express:21.1.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:application_performance_management:13.4.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:application_performance_management:13.5.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:application_testing_suite:13.3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_analytics:8.2.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_analytics:8.2.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_analytics:8.2.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_analytics:8.21:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_insight:8.2.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_insight:8.2.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_insight:8.2.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_safety:8.2.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_safety:8.2.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:argus_safety:8.2.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_apis:18.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_apis:18.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_apis:18.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_apis:19.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_apis:19.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_apis:20.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_apis:21.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_deposits_and_lines_of_credit_servicing:2.12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_digital_experience:17.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_digital_experience:18.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_digital_experience:18.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_digital_experience:19.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_digital_experience:19.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_digital_experience:20.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_digital_experience:21.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_enterprise_default_management:2.6.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_enterprise_default_management:2.7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_enterprise_default_management:2.7.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_enterprise_default_management:2.10.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_enterprise_default_management:2.12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_enterprise_default_managment:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_loans_servicing:2.12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_party_management:2.7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_platform:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_platform:2.6.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_platform:2.7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:banking_platform:2.7.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:bi_publisher:5.5.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:bi_publisher:11.1.1.9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:bi_publisher:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:bi_publisher:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:big_data_spatial_and_graph:23.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:business_activity_monitoring:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:business_intelligence:5.5.0.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:business_intelligence:5.9.0.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:business_intelligence:12.2.1.3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:business_intelligence:12.2.1.4.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:business_process_management_suite:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:business_process_management_suite:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:clinical:5.2.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:clinical:5.2.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:commerce_guided_search:11.3.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:commerce_platform:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_application_session_controller:3.9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_billing_and_revenue_management:12.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_billing_and_revenue_management:12.0.0.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_billing_and_revenue_management_elastic_charging_engine:11.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_billing_and_revenue_management_elastic_charging_engine:12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_calendar_server:8.0.0.5.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_calendar_server:8.0.0.6.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_automated_test_suite:1.8.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_binding_support_function:1.9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_binding_support_function:1.10.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_console:1.7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_network_function_cloud_native_environment:1.9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_network_repository_function:1.14.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_policy:1.14.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_security_edge_protection_proxy:1.5.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_security_edge_protection_proxy:1.6.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_security_edge_protection_proxy:1.15.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_service_communication_proxy:1.14.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_unified_data_repository:1.14.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_contacts_server:8.0.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_converged_application_server_-_service_controller:6.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_convergence:3.0.2.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_convergent_charging_controller:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_convergent_charging_controller:6.0.1.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_data_model:11.3.2.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_data_model:11.3.2.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_data_model:11.3.2.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_data_model:12.1.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_data_model:12.1.2.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_design_studio:7.3.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_design_studio:7.3.5:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_design_studio:7.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_design_studio:7.4.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_design_studio:7.4.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_diameter_signaling_route:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_eagle_application_processor:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_instant_messaging_server:10.0.1.5.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_interactive_session_recorder:6.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_interactive_session_recorder:6.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_messaging_server:8.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_metasolv_solution:6.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_network_charging_and_control:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_network_charging_and_control:6.0.1.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_network_integrity:7.3.5:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_network_integrity:7.3.6:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_offline_mediation_controller:12.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_operations_monitor:3.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_operations_monitor:4.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_operations_monitor:4.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_operations_monitor:4.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_operations_monitor:5.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_pricing_design_center:12.0.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_pricing_design_center:12.0.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_service_broker:6.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_services_gatekeeper:7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_session_border_controller:8.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_session_border_controller:8.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_session_border_controller:8.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_session_border_controller:9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_unified_inventory_management:7.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_unified_inventory_management:7.3.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_unified_inventory_management:7.3.5:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_unified_inventory_management:7.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_unified_inventory_management:7.4.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_unified_inventory_management:7.4.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_unified_inventory_management:7.5.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_webrtc_session_controller:7.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_webrtc_session_controller:7.2.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:data_integrator:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:data_integrator:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:database_server:12.1.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:database_server:12.1.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:database_server:19c:*:*:*:*:*:*:*|cpe:2.3:a:oracle:database_server:21c:*:*:*:*:*:*:*|cpe:2.3:a:oracle:demantra_demand_management:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:documaker:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:e-business_suite:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_communications_broker:3.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_data_quality:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_data_quality:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_manager_base_platform:13.4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_manager_base_platform:13.5.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_manager_ops_center:12.4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_session_border_controller:8.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_session_border_controller:9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:essbase:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:essbase:11.1.2.4.47:*:*:*:*:*:*:*|cpe:2.3:a:oracle:essbase_administration_services:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:essbase_administration_services:11.1.2.4.47:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_analytical_applications_infrastructure:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_analytical_applications_infrastructure:7.3.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_behavior_detection_platform:8.0.7:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_behavior_detection_platform:8.0.8:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_behavior_detection_platform:8.0.11:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_enterprise_case_management:8.0.7:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_enterprise_case_management:8.0.8:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_enterprise_case_management:8.0.11:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_foreign_account_tax_compliance_act_management:8.0.7:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_foreign_account_tax_compliance_act_management:8.0.8:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_foreign_account_tax_compliance_act_management:8.0.11:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_model_management_and_governance:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:financial_services_trade-based_anti_money_laundering:8.0.7:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:financial_services_trade-based_anti_money_laundering:8.0.8:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:flexcube_investor_servicing:12.0.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:flexcube_investor_servicing:12.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:flexcube_investor_servicing:12.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:flexcube_investor_servicing:12.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:flexcube_investor_servicing:14.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:flexcube_investor_servicing:14.5.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:flexcube_private_banking:12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:flexcube_private_banking:12.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:fusion_middleware:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:fusion_middleware:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:fusion_middleware_mapviewer:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:goldengate:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:goldengate_application_adapters:19.1.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:graalvm:20.3.4:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:graalvm:21.3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:graph_server_and_client:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:health_sciences_clinical_development_analytics:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:health_sciences_inform_crf_submit:6.2.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:health_sciences_information_manager:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:health_sciences_information_manager:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:healthcare_data_repository:7.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:healthcare_data_repository:8.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:healthcare_data_repository:8.1.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:healthcare_foundation:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:healthcare_foundation:8.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:healthcare_foundation:8.1.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:healthcare_translational_research:4.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_cruise_shipboard_property_management_system:20.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_opera_5_property_services:5.6:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_reporting_and_analytics:9.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_suite8:8.10.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_suite8:8.11.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_suite8:8.12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_suite8:8.13.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hospitality_suite8:8.14.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hyperion_financial_management:11.1.2.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hyperion_financial_management:11.2.6.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hyperion_ilearning:6.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hyperion_ilearning:6.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:hyperion_infrastructure_technology:11.2.7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:instantis_enterprisetrack:17.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:instantis_enterprisetrack:17.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:instantis_enterprisetrack:17.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_data_gateway:11.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_data_gateway:11.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_data_gateway:11.2.7:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_data_gateway:11.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_data_gateway:11.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_insbridge_rating_and_underwriting:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_insbridge_rating_and_underwriting:5.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration:11.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration:11.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration:11.2.7:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration:11.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration:11.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration_j2ee:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration_j2ee:10.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration_j2ee:10.2.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_policy_administration_j2ee:11.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_rules_palette:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_rules_palette:10.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_rules_palette:10.2.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_rules_palette:11.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:insurance_rules_palette:11.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:java_se:7u321:*:*:*:*:*:*:*|cpe:2.3:a:oracle:java_se:8u311:*:*:*:*:*:*:*|cpe:2.3:a:oracle:java_se:17.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:jd_edwards_enterpriseone_orchestrator:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:jdk:11.0.13:*:*:*:*:*:*:*|cpe:2.3:a:oracle:managed_file_transfer:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:managed_file_transfer:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:mysql_cluster:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:mysql_connectors:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:mysql_connectors:8.0.27:*:*:*:*:*:*:*|cpe:2.3:a:oracle:mysql_server:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:mysql_server:5.7.36:*:*:*:*:*:*:*|cpe:2.3:a:oracle:mysql_workbench:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:nosql_database:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:oss_support_tools:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_cs_sa_integration_pack:9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_cs_sa_integration_pack:9.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_people_tools:8.57:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_people_tools:8.58:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_people_tools:8.59:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.57:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.58:*:*:*:*:*:*:*|cpe:2.3:a:oracle:policy_automation:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:policy_automation:10.4.7:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_analytics:18.8.3.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_analytics:19.12.11.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_analytics:20.12.12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_data_warehouse:18.8.3.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_data_warehouse:19.12.11.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_data_warehouse:20.12.12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_gateway:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_gateway:21.12.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_p6_enterprise_project_portfolio_management:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_p6_enterprise_project_portfolio_management:21.12.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_p6_professional_project_management:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_portfolio_management:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_portfolio_management:20.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_portfolio_management:20.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_unifier:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_unifier:18.8:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_unifier:19.12:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_unifier:20.12:*:*:*:*:*:*:*|cpe:2.3:a:oracle:primavera_unifier:21.12:*:*:*:*:*:*:*|cpe:2.3:a:oracle:rapid_planning:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:real-time_decision_server:3.2.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:real_user_experience_insight:13.4.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:real_user_experience_insight:13.5.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:rest_data_services:21.2.4:*:*:*:-:*:*:*|cpe:2.3:a:oracle:retail_allocation:14.1.3.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_allocation:15.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_allocation:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_allocation:19.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_analytics:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_assortment_planning:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_back_office:14.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_central_office:14.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_customer_insights:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_customer_management_and_segmentation_foundation:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_eftlink:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_eftlink:17.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_eftlink:18.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_eftlink:19.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_eftlink:20.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_extract_transform_and_load:13.2.8:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_financial_integration:14.1.3.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_financial_integration:15.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_financial_integration:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_financial_integration:19.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_fiscal_management:14.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_integration_bus:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_integration_bus:13.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_integration_bus:14.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_integration_bus:14.1.3.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_integration_bus:15.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_integration_bus:19.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_integration_bus:19.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_invoice_matching:15.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_invoice_matching:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_merchandising_system:19.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_order_broker:16.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_order_broker:18.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_order_broker:19.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_order_management_system:19.5:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_point-of-sale:14.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:14.1.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:14.1.3.46:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:15.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:15.0.3.115:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:16.0.3.240:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:13.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:14.0.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:14.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:14.1.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:15.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:15.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:16.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_price_management:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_returns_management:14.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_service_backbone:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_service_backbone:14.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_service_backbone:14.1.3.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_service_backbone:15.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_service_backbone:19.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_service_backbone:19.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_size_profile_optimization:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_xstore_point_of_service:17.0.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_xstore_point_of_service:18.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_xstore_point_of_service:19.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_xstore_point_of_service:20.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:sd-wan_aware:8.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:sd-wan_edge:9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:sd-wan_edge:9.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:secure_backup:18.1.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:siebel_applications:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:spatial_studio:21.2.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:thesaurus_management_system:5.2.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:thesaurus_management_system:5.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:thesaurus_management_system:5.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:timesten_in-memory_database:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_framework:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_framework:4.2.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_framework:4.2.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_framework:4.4.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_framework:4.4.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_framework:4.4.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_testing_accelerator:6.0.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_testing_accelerator:6.0.0.2.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:utilities_testing_accelerator:6.0.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:vm_virtualbox:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:webcenter_portal:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:webcenter_portal:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:12.1.3.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:14.1.1.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:zfs_storage_appliance_kit:8.8:*:*:*:*:*:*:*|cpe:2.3:a:oracle:zfs_storage_application_integration_engineering_software:1.3.3:*:*:*:*:*:*:*|cpe:2.3:o:oracle:communications_messaging_server:8.1:*:*:*:*:*:*:*|cpe:2.3:o:oracle:solaris:10:*:*:*:*:*:*:*|cpe:2.3:o:oracle:solaris:11:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m10-1_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m10-4_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m10-4s_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m12-1_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m12-2_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m12-2s_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m12-2s:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1356,8 +1473,10 @@
       <c r="D28" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E28" t="n">
-        <v>3.1</v>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1369,8 +1488,11 @@
           <t>cpe:2.3:o:fujitsu:eternus_cs8000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:eternus_cs8000_firmware:8.1:-:*:*:*:*:*:*|cpe:2.3:h:fujitsu:eternus_cs8000:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1391,8 +1513,10 @@
       <c r="D29" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E29" t="n">
-        <v>3.1</v>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1404,8 +1528,11 @@
           <t>cpe:2.3:o:fujitsu:eternus_cs8000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:eternus_cs8000_firmware:8.1:-:*:*:*:*:*:*|cpe:2.3:h:fujitsu:eternus_cs8000:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1426,8 +1553,10 @@
       <c r="D30" t="n">
         <v>7.8</v>
       </c>
-      <c r="E30" t="n">
-        <v>3.1</v>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1439,8 +1568,11 @@
           <t>cpe:2.3:a:fujitsu:plugfree_network:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1461,8 +1593,10 @@
       <c r="D31" t="n">
         <v>7.8</v>
       </c>
-      <c r="E31" t="n">
-        <v>3.1</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1474,8 +1608,11 @@
           <t>cpe:2.3:o:fujitsu:lifebook_a3510_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_a3510:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9310_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9310:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7511_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7511:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7411_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7411:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7311_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7311:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9311_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9311:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5510_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5510:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7510_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7510:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7410_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7410:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7310_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7310:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e459_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e459:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e449_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e449:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1498,8 +1635,10 @@
       <c r="D32" t="n">
         <v>5.5</v>
       </c>
-      <c r="E32" t="n">
-        <v>3.1</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1511,8 +1650,11 @@
           <t>cpe:2.3:a:daikinlatam:svmpc1:*:*:*:*:*:*:*:*|cpe:2.3:a:daikinlatam:svmpc2:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>daikin</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1533,8 +1675,10 @@
       <c r="D33" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E33" t="n">
-        <v>3.1</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1546,8 +1690,11 @@
           <t>cpe:2.3:a:daikinlatam:svmpc1:*:*:*:*:*:*:*:*|cpe:2.3:a:daikinlatam:svmpc2:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>daikin</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1568,8 +1715,10 @@
       <c r="D34" t="n">
         <v>7.4</v>
       </c>
-      <c r="E34" t="n">
-        <v>3.1</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1581,8 +1730,11 @@
           <t>cpe:2.3:a:fujitsu:tsclinical_define.xml_generator:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:tsclinical_metadata_desktop_tools:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1603,8 +1755,10 @@
       <c r="D35" t="n">
         <v>6.3</v>
       </c>
-      <c r="E35" t="n">
-        <v>3.1</v>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1616,8 +1770,11 @@
           <t>cpe:2.3:o:google:android:*:*:*:*:*:*:*:*|cpe:2.3:h:lg:v60_thin_q_5g:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>lg thinq</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1638,8 +1795,10 @@
       <c r="D36" t="n">
         <v>2.7</v>
       </c>
-      <c r="E36" t="n">
-        <v>3.1</v>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1647,8 +1806,11 @@
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1690,8 +1852,10 @@
       <c r="D37" t="n">
         <v>5.5</v>
       </c>
-      <c r="E37" t="n">
-        <v>3.1</v>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
@@ -1699,8 +1863,11 @@
           <t>cpe:2.3:o:linux:linux_kernel:*:*:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.10:rc1:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.10:rc2:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.10:rc3:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>friedrich</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1721,8 +1888,10 @@
       <c r="D38" t="n">
         <v>6.5</v>
       </c>
-      <c r="E38" t="n">
-        <v>3.1</v>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1734,8 +1903,11 @@
           <t>cpe:2.3:o:fujitsu:network_edgiot_gw1500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:network_edgiot_gw1500:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1756,8 +1928,10 @@
       <c r="D39" t="n">
         <v>8.4</v>
       </c>
-      <c r="E39" t="n">
-        <v>3.1</v>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1765,8 +1939,11 @@
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1787,8 +1964,10 @@
       <c r="D40" t="n">
         <v>5.1</v>
       </c>
-      <c r="E40" t="n">
-        <v>2</v>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
@@ -1796,8 +1975,11 @@
           <t>cpe:2.3:a:fujitsu:chocoa:1.0beta7r:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1818,8 +2000,10 @@
       <c r="D41" t="n">
         <v>7.5</v>
       </c>
-      <c r="E41" t="n">
-        <v>2</v>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
@@ -1827,8 +2011,11 @@
           <t>cpe:2.3:a:fujitsu:serverview:2.50:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:3.60l98:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:3.60l99:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.10l11:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.11l11b:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.11l81:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.4:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.5:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.6:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.7:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.8:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.9:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.10:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.11:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.12:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.30.13:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.40.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.40.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.40.3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.40.4:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.40.5:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.40.6:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.4:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.5:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.6:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.7:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview:4.50.8:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1849,8 +2036,10 @@
       <c r="D42" t="n">
         <v>5</v>
       </c>
-      <c r="E42" t="n">
-        <v>2</v>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
@@ -1858,8 +2047,11 @@
           <t>cpe:2.3:h:fujitsu:primergy_bx300:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1880,8 +2072,10 @@
       <c r="D43" t="n">
         <v>5</v>
       </c>
-      <c r="E43" t="n">
-        <v>2</v>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1893,8 +2087,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus_developer:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:plus:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.1:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.1:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.2:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.2:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.3:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.3:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0a:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0a:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks:7.0:*:modelers_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks:8.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks:8.0:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:8.01:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:8.01:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.0:*:standard_j:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1915,8 +2112,10 @@
       <c r="D44" t="n">
         <v>10</v>
       </c>
-      <c r="E44" t="n">
-        <v>2</v>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1928,8 +2127,11 @@
           <t>cpe:2.3:a:fujitsu-siemens:webtransactions:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu-siemens:webtransactions:7.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1950,8 +2152,10 @@
       <c r="D45" t="n">
         <v>4.3</v>
       </c>
-      <c r="E45" t="n">
-        <v>2</v>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1963,8 +2167,11 @@
           <t>cpe:2.3:a:fujitsu-siemens:webtransactions:6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu-siemens:webtransactions:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu-siemens:webtransactions:7.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1985,8 +2192,10 @@
       <c r="D46" t="n">
         <v>10</v>
       </c>
-      <c r="E46" t="n">
-        <v>2</v>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -1998,8 +2207,11 @@
           <t>cpe:2.3:a:fujitsu:systemcastwizard_lite:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.7:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.8:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.8a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.9:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:2.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2020,8 +2232,10 @@
       <c r="D47" t="n">
         <v>10</v>
       </c>
-      <c r="E47" t="n">
-        <v>2</v>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2033,8 +2247,11 @@
           <t>cpe:2.3:a:fujitsu:systemcastwizard_lite:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.7:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.8:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.8a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.9:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:2.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2055,8 +2272,10 @@
       <c r="D48" t="n">
         <v>5</v>
       </c>
-      <c r="E48" t="n">
-        <v>2</v>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2068,8 +2287,11 @@
           <t>cpe:2.3:a:fujitsu:systemcastwizard_lite:1.7:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.8:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.8a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:1.9:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:2.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemcastwizard_lite:2.0a:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2090,8 +2312,10 @@
       <c r="D49" t="n">
         <v>5</v>
       </c>
-      <c r="E49" t="n">
-        <v>2</v>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2103,8 +2327,11 @@
           <t>cpe:2.3:a:fujitsu:enhanced_support_facility:3.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:enhanced_support_facility:3.0.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2125,8 +2352,10 @@
       <c r="D50" t="n">
         <v>6.8</v>
       </c>
-      <c r="E50" t="n">
-        <v>2</v>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2138,8 +2367,11 @@
           <t>cpe:2.3:a:fujitsu:jasmine2000:*:enterprise:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows:*:*:*:*:*:*:*:*|cpe:2.3:o:sun:solaris:7:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2160,8 +2392,10 @@
       <c r="D51" t="n">
         <v>10</v>
       </c>
-      <c r="E51" t="n">
-        <v>2</v>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2173,8 +2407,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server:9.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.2.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:10.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.2.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:10.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2195,8 +2432,10 @@
       <c r="D52" t="n">
         <v>7.5</v>
       </c>
-      <c r="E52" t="n">
-        <v>3</v>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2208,8 +2447,11 @@
           <t>cpe:2.3:o:oracle:fujitsu_m10_firmware:*:*:*:*:*:*:*:*|cpe:2.3:a:intel:intelligent_platform_management_interface:2.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2230,8 +2472,10 @@
       <c r="D53" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E53" t="n">
-        <v>3.1</v>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2243,8 +2487,11 @@
           <t>cpe:2.3:a:apache:archiva:*:*:*:*:*:*:*:*|cpe:2.3:a:apache:archiva:1.2:-:*:*:*:*:*:*|cpe:2.3:a:apache:archiva:1.2.2:*:*:*:*:*:*:*|cpe:2.3:a:apache:struts:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_business_process_manager_analytics:12.0:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_server_2003:-:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_server_2008:-:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_business_process_manager_analytics:12.1:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_server_2012:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:solaris:11:*:*:*:*:*:*:*|cpe:2.3:a:oracle:siebel_apps_-_e-billing:6.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:siebel_apps_-_e-billing:6.1.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:siebel_apps_-_e-billing:6.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2265,8 +2512,10 @@
       <c r="D54" t="n">
         <v>5.9</v>
       </c>
-      <c r="E54" t="n">
-        <v>3.1</v>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2278,8 +2527,11 @@
           <t>cpe:2.3:a:oracle:communications_application_session_controller:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:11.1.1.7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:11.1.1.9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.1.3.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.2.1.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.2.1.2.0:*:*:*:*:*:*:*|cpe:2.3:o:oracle:integrated_lights_out_manager_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m3000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m3000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m4000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m4000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m5000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m5000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m8000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m8000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m9000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m9000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:12.04:*:*:*:esm:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:12.10:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:13.04:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:13.10:*:*:*:*:*:*:*|cpe:2.3:a:mozilla:firefox:*:*:*:*:*:*:*:*|cpe:2.3:a:mozilla:seamonkey:*:*:*:*:*:*:*:*|cpe:2.3:a:mozilla:thunderbird:*:*:*:*:*:*:*:*|cpe:2.3:a:mozilla:thunderbird_esr:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2300,8 +2552,10 @@
       <c r="D55" t="n">
         <v>4.3</v>
       </c>
-      <c r="E55" t="n">
-        <v>2</v>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2313,8 +2567,11 @@
           <t>cpe:2.3:a:fujitsu:serverview_operations_manager:5.00.09:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:serverview_operations_manager:6.30.05:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2335,8 +2592,10 @@
       <c r="D56" t="n">
         <v>3.7</v>
       </c>
-      <c r="E56" t="n">
-        <v>3.1</v>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2348,8 +2607,11 @@
           <t>cpe:2.3:a:oracle:communications_application_session_controller:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_policy_management:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:11.1.1.7.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:11.1.1.9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.1.3.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.2.1.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:http_server:12.2.1.2.0:*:*:*:*:*:*:*|cpe:2.3:o:oracle:integrated_lights_out_manager_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:7.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:a:redhat:satellite:5.7:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_desktop:5.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_desktop:6.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_desktop:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:6.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:7.1:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:7.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:7.3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:7.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:7.5:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:7.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:7.7:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server:5.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server:6.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:6.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.7:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:7.3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:7.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:7.7:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_workstation:5.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_workstation:6.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_workstation:7.0:*:*:*:*:*:*:*|cpe:2.3:a:suse:linux_enterprise_debuginfo:11:sp3:*:*:*:*:*:*|cpe:2.3:a:suse:linux_enterprise_debuginfo:11:sp4:*:*:*:*:*:*|cpe:2.3:o:opensuse:opensuse:13.1:*:*:*:*:*:*:*|cpe:2.3:o:opensuse:opensuse:13.2:*:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_desktop:11:sp3:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_desktop:11:sp4:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_desktop:12:-:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:10:sp4:*:*:ltss:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:11:sp1:*:*:ltss:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:11:sp2:*:*:ltss:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:11:sp3:*:*:*:vmware:*:*|cpe:2.3:o:suse:linux_enterprise_server:12:-:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_software_development_kit:11:sp3:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_software_development_kit:12:-:*:*:*:*:*:*|cpe:2.3:a:suse:manager:1.7:*:*:*:*:*:*:*|cpe:2.3:o:suse:linux_enterprise_server:11:sp2:*:*:*:-:*:*|cpe:2.3:o:canonical:ubuntu_linux:12.04:*:*:*:esm:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:14.04:*:*:*:esm:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:15.04:*:*:*:*:*:*:*|cpe:2.3:a:redhat:satellite:5.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:5.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:6.0:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m3000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m3000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m4000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m4000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m5000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m5000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m8000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m8000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m9000_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m9000:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:e6000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:e6000:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:e9000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:e9000:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_18500_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_18500:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_18800_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_18800:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_18800f_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_18800f:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_9000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_9000:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_cse_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_cse:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_hvs85t_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_hvs85t:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_s2600t_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_s2600t:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_s5500t_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_s5500t:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_s5600t_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_s5600t:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_s5800t_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_s5800t:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_s6800t_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_s6800t:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:oceanstor_vis6600t_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:oceanstor_vis6600t:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:quidway_s9300_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:quidway_s9300:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s7700_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s7700:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:9700_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:9700:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s12700_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s12700:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s2700_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s2700:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s3700_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s3700:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5700ei_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5700ei:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5700hi_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5700hi:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5700si_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5700si:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5710ei_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5710ei:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5710hi_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5710hi:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s6700_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s6700:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s2750_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s2750:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5700li_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5700li:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5700s-li_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5700s-li:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5720hi_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5720hi:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:s5720ei_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:s5720ei:-:*:*:*:*:*:*:*|cpe:2.3:o:huawei:te60_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:huawei:te60:-:*:*:*:*:*:*:*|cpe:2.3:a:huawei:oceanstor_replicationdirector:v100r003c00:*:*:*:*:*:*:*|cpe:2.3:a:huawei:policy_center:v100r003c00:*:*:*:*:*:*:*|cpe:2.3:a:huawei:policy_center:v100r003c10:*:*:*:*:*:*:*|cpe:2.3:a:huawei:smc2.0:v100r002c01:*:*:*:*:*:*:*|cpe:2.3:a:huawei:smc2.0:v100r002c02:*:*:*:*:*:*:*|cpe:2.3:a:huawei:smc2.0:v100r002c03:*:*:*:*:*:*:*|cpe:2.3:a:huawei:smc2.0:v100r002c04:*:*:*:*:*:*:*|cpe:2.3:a:huawei:ultravr:v100r003c00:*:*:*:*:*:*:*|cpe:2.3:a:ibm:cognos_metrics_manager:10.1:*:*:*:*:*:*:*|cpe:2.3:a:ibm:cognos_metrics_manager:10.1.1:*:*:*:*:*:*:*|cpe:2.3:a:ibm:cognos_metrics_manager:10.2:*:*:*:*:*:*:*|cpe:2.3:a:ibm:cognos_metrics_manager:10.2.1:*:*:*:*:*:*:*|cpe:2.3:a:ibm:cognos_metrics_manager:10.2.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2370,8 +2632,10 @@
       <c r="D57" t="n">
         <v>3.7</v>
       </c>
-      <c r="E57" t="n">
-        <v>3</v>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2383,8 +2647,11 @@
           <t>cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.0.2:*:*:*:*:*:*:*|cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.5.1:*:*:*:*:*:*:*|cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.5.2:*:*:*:*:*:*:*|cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.5.3:*:*:*:*:*:*:*|cpe:2.3:a:nttdata:terasoluna_server_framework_for_java_web:2.0.6.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2405,8 +2672,10 @@
       <c r="D58" t="n">
         <v>7.5</v>
       </c>
-      <c r="E58" t="n">
-        <v>3.1</v>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2418,8 +2687,11 @@
           <t>cpe:2.3:a:openssl:openssl:*:*:*:*:*:*:*:*|cpe:2.3:a:openssl:openssl:0.9.8:*:*:*:*:*:*:*|cpe:2.3:a:openssl:openssl:1.0.1:*:*:*:*:*:*:*|cpe:2.3:a:openssl:openssl:1.1.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_desktop:6.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_desktop:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server:6.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:7.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_eus:7.3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_eus:7.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_eus:7.5:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_eus:7.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:7.3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:7.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_workstation:6.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_workstation:7.0:*:*:*:*:*:*:*|cpe:2.3:a:redhat:jboss_enterprise_application_platform:6.0.0:*:*:*:*:*:*:*|cpe:2.3:a:redhat:jboss_enterprise_application_platform:6.4.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:6.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:7.0:*:*:*:*:*:*:*|cpe:2.3:o:netapp:cn1610_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:cn1610:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:clustered_data_ontap_antivirus_connector:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:data_ontap:-:*:*:*:*:7-mode:*:*|cpe:2.3:a:netapp:data_ontap_edge:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:e-series_santricity_os_controller:*:*:*:*:*:*:*:*|cpe:2.3:a:netapp:host_agent:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:oncommand_balance:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:oncommand_unified_manager:-:*:*:*:*:7-mode:*:*|cpe:2.3:a:netapp:oncommand_workflow_automation:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:ontap_select_deploy:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:service_processor:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:smi-s_provider:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:snapcenter_server:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:snapdrive:-:*:*:*:*:unix:*:*|cpe:2.3:a:netapp:storagegrid:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:storagegrid_webscale:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:clustered_data_ontap:-:*:*:*:*:*:*:*|cpe:2.3:o:paloaltonetworks:pan-os:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:adaptive_access_manager:11.1.2.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:application_testing_suite:13.3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_analytics:12.1.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_ip_service_activator:7.3.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_ip_service_activator:7.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:core_rdbms:11.2.0.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:core_rdbms:12.1.0.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:core_rdbms:12.2.0.1:*:*:*:*:*:*:*|cpe:2.3:a:oracle:core_rdbms:18c:*:*:*:*:*:*:*|cpe:2.3:a:oracle:core_rdbms:19c:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_manager_ops_center:12.3.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_manager_ops_center:12.4.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:goldengate_application_adapters:12.3.2.1.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:jd_edwards_enterpriseone_tools:9.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.56:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.57:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.58:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:15.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:retail_predictive_application_server:16.0.3:*:*:*:*:*:*:*|cpe:2.3:a:oracle:timesten_in-memory_database:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:10.3.6.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:12.1.3.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:12.2.1.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:weblogic_server:12.2.1.4.0:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2440,8 +2712,10 @@
       <c r="D59" t="n">
         <v>7.5</v>
       </c>
-      <c r="E59" t="n">
-        <v>3.1</v>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -2449,8 +2723,11 @@
           <t>cpe:2.3:a:ntp:ntp:*:*:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:-:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta4:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta5:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-rc1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-rc2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p10:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2-rc1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2-rc2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2-rc3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3-rc1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3-rc2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3-rc3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p4:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p5:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p6:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p7:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p8:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p9:*:*:*:*:*:*|cpe:2.3:a:synology:router_manager:*:*:*:*:*:*:*:*|cpe:2.3:a:synology:skynas:*:*:*:*:*:*:*:*|cpe:2.3:a:synology:virtual_diskstation_manager:*:*:*:*:*:*:*:*|cpe:2.3:o:synology:diskstation_manager:*:*:*:*:*:*:*:*|cpe:2.3:o:synology:vs960hd_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:synology:vs960hd:-:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:12.04:*:*:*:esm:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:14.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:16.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:17.10:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.04:*:*:*:lts:*:*:*|cpe:2.3:a:netapp:hci:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:solidfire:-:*:*:*:*:*:*:*|cpe:2.3:a:hpe:hpux-ntp:*:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:fujitsu_m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:oracle:fujitsu_m12-2s:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2471,8 +2748,10 @@
       <c r="D60" t="n">
         <v>7.8</v>
       </c>
-      <c r="E60" t="n">
-        <v>3</v>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -2484,8 +2763,11 @@
           <t>cpe:2.3:a:portrait:portrait_display_sdk:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:displayview_click:6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:displayview_click:6.01:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:displayview_click_suite:5.0:*:*:*:*:*:*:*|cpe:2.3:a:hp:display_assistant:2.1:*:*:*:*:*:*:*|cpe:2.3:a:hp:my_display:2.0:*:*:*:*:*:*:*|cpe:2.3:a:philips:smart_control_premium:2.23:*:*:*:*:*:*:*|cpe:2.3:a:philips:smart_control_premium:2.25:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2506,8 +2788,10 @@
       <c r="D61" t="n">
         <v>5.3</v>
       </c>
-      <c r="E61" t="n">
-        <v>3.1</v>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -2519,8 +2803,11 @@
           <t>cpe:2.3:a:openbsd:openssh:*:*:*:*:*:*:*:*|cpe:2.3:a:winscp:winscp:*:*:*:*:*:*:*:*|cpe:2.3:a:netapp:cloud_backup:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:element_software:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:ontap_select_deploy:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:steelstore_cloud_integrated_storage:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:storage_automation_store:-:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:9.0:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:14.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:16.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.10:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:7.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:8.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.1:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_eus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_aus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.4:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux_server_tus:8.6:*:*:*:*:*:*:*|cpe:2.3:o:oracle:solaris:10:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:o:siemens:scalance_x204rna_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:siemens:scalance_x204rna:-:*:*:*:*:*:*:*|cpe:2.3:o:siemens:scalance_x204rna_eec_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:siemens:scalance_x204rna_eec:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2541,8 +2828,10 @@
       <c r="D62" t="n">
         <v>9.6</v>
       </c>
-      <c r="E62" t="n">
-        <v>3</v>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -2550,8 +2839,11 @@
           <t>cpe:2.3:o:fujitsu:lx901_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lx901:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:gk900_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:gk900:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2572,8 +2864,10 @@
       <c r="D63" t="n">
         <v>7.8</v>
       </c>
-      <c r="E63" t="n">
-        <v>3.1</v>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -2585,8 +2879,11 @@
           <t>cpe:2.3:a:fujitsu:paperstream_ip_\(twain\):1.42.0.5685:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2607,8 +2904,10 @@
       <c r="D64" t="n">
         <v>6.6</v>
       </c>
-      <c r="E64" t="n">
-        <v>3.1</v>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2620,8 +2919,11 @@
           <t>cpe:2.3:o:fujitsu:lx390_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lx390:gk381:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2642,8 +2944,10 @@
       <c r="D65" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E65" t="n">
-        <v>3.1</v>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
@@ -2651,8 +2955,11 @@
           <t>cpe:2.3:o:fujitsu:lx390_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lx390:gk381:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2673,8 +2980,10 @@
       <c r="D66" t="n">
         <v>7.5</v>
       </c>
-      <c r="E66" t="n">
-        <v>3.1</v>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2686,8 +2995,11 @@
           <t>cpe:2.3:o:fujitsu:lx390_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lx390:gk381:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2708,8 +3020,10 @@
       <c r="D67" t="n">
         <v>5.9</v>
       </c>
-      <c r="E67" t="n">
-        <v>3.1</v>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2721,8 +3035,11 @@
           <t>cpe:2.3:o:fujitsu:gp7000f_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:gp7000f:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primepower_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primepower:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:gps_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:gps:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m3000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m3000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m4000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m4000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m5000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m5000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m8000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m8000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_enterprise_m9000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_enterprise_m9000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_m12-1_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_m12-2_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sparc_m12-2s_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sparc_m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2530_m5_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2530_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2540_m5_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2540_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx4770_m5_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx4770_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx2550_m5_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx2550_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:granpower_5000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:granpower_5000:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primequest_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primequest:-:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.0a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.1.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.1.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.2:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.2:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3.1a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3.1a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.1:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.3:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.3:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.0b:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.1.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.1.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.1.0b:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.1.0b:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.2.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.2.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.2.0a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.2.0a:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:10.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:10.0.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:10.1.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:10.1.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.0.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:12.0.0:*:*:*:enterprise:*:x86:*|cpe:2.3:a:fujitsu:interstage_application_server:12.0.0:*:*:*:standard-j:*:x86:*|cpe:2.3:a:fujitsu:interstage_application_server:12.1.0:*:*:*:enterprise:*:x86:*|cpe:2.3:a:fujitsu:interstage_application_server:12.1.0:*:*:*:standard-j:*:x86:*|cpe:2.3:a:fujitsu:interstage_application_server:12.2.0:*:*:*:enterprise:*:x86:*|cpe:2.3:a:fujitsu:interstage_application_server:12.2.0:*:*:*:standard-j:*:x86:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l10:*:*:*:developer:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l10:*:*:*:enterprise:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l10:*:*:*:standard:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l20:*:*:*:developer:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l20:*:*:*:enterprise:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l20:*:*:*:standard:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l21:*:*:*:enterprise:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.0l21:*:*:*:standard:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.1:*:*:*:developer:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.1:*:*:*:enterprise:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:1.1:*:*:*:standard:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:2.0.0:*:*:*:developer:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:2.0.1:*:*:*:developer:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:2.0.1:*:*:*:enterprise:.net:*:*|cpe:2.3:a:fujitsu:interstage_business_application_manager:2.0.1:*:*:*:standard:.net:*:*|cpe:2.3:a:fujitsu:interstage_list_works:9.0.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:9.0.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:9.0.1a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:9.0.1a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.0.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.1.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.1.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.2.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.2.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0b:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0b:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0c:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.0c:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.2:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.2:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.2a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_list_works:10.3.2a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.1.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.1.0b:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:9.2.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:10.0.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:10.1.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:11.0.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:11.1.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:11.1.0a:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_studio:12.0.0:*:*:*:standard-j:*:x86:*|cpe:2.3:a:fujitsu:interstage_studio:12.1.0:*:*:*:standard-j:*:x86:*|cpe:2.3:a:fujitsu:interstage_studio:12.2.0:*:*:*:standard-j:*:x86:*|cpe:2.3:a:fujitsu:interstage_web_server_express:11.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_web_server_express:11.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:linkexpress:v5.0l20:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:serverview_resource_orchestrator:3.0.0:*:*:*:cloud:*:*:*|cpe:2.3:a:fujitsu:serverview_resource_orchestrator:3.1.0:*:*:*:cloud:*:*:*|cpe:2.3:a:fujitsu:serverview_resource_orchestrator:3.1.1:*:*:*:cloud:*:*:*|cpe:2.3:a:fujitsu:serverview_resource_orchestrator:3.1.2:*:*:*:cloud:*:*:*|cpe:2.3:a:fujitsu:serverview_resource_orchestrator:3.2.0:*:*:*:cloud:*:*:*|cpe:2.3:a:fujitsu:serverview_resource_orchestrator:3.3.0:*:*:*:cloud:*:*:*|cpe:2.3:a:fujitsu:serverview_resource_orchestrator:3.4.0:*:*:*:cloud:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.0.0b:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.0.1a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.0.1b:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.0e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.1e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.2e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.1.3e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.2.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.2.0e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_keeper:15.3.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.0.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.0.1a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.0.1b:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.1.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.1.0e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.1.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.1.1e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.1.3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.1.3e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.2.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.2.0e:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.3.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_patrol:15.3.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.0.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.0.0a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.0.0a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.1.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.1.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.1.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_it_change_manager_v14g:14.1.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.0b:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.0b:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.6.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.6.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.6.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.6.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.7.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.7.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0e:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0e:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.0.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.1.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.1.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.1.2a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.1.3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation:15.1.3a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation_v14g:14.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_runbook_automation_v14g:14.1.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_software_configuration_manager:15.5.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_software_configuration_manager_express:15.5.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:triole_cloud_middle_set_b_set:1.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:triole_cloud_middle_set_b_set:1.1.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:triole_cloud_middle_set_b_set:1.1.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:triole_cloud_middle_set_b_set:1.1.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:triole_cloud_middle_set_b_set:1.2.0:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:datacenter:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:datacenter_without_hyper-v:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:enterprise:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:enterprise_without_hyper-v:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:foundation:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:standard:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:standard_without_hyper-v:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:datacenter:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:enterprise:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:foundation:*:x86:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:standard:*:x86:*|cpe:2.3:o:microsoft:windows_server_2012:-:*:*:*:datacenter:*:x86:*|cpe:2.3:o:microsoft:windows_server_2012:-:*:*:*:foundation:*:x86:*|cpe:2.3:o:microsoft:windows_server_2012:-:*:*:*:standard:*:x86:*|cpe:2.3:o:microsoft:windows_server_2012:r2:*:*:*:datacenter:*:x64:*|cpe:2.3:o:microsoft:windows_server_2012:r2:*:*:*:foundation:*:x64:*|cpe:2.3:o:microsoft:windows_server_2012:r2:*:*:*:standard:*:x64:*|cpe:2.3:o:microsoft:windows_server_2016:-:*:*:*:datacenter:*:x86:*|cpe:2.3:o:microsoft:windows_server_2016:-:*:*:*:standard:*:x86:*|cpe:2.3:o:microsoft:windows_server_2019:-:*:*:*:datacenter:*:x86:*|cpe:2.3:o:microsoft:windows_server_2019:-:*:*:*:standard:*:x86:*|cpe:2.3:o:microsoft:windows_small_business_server_2011:-:*:*:*:essentials:*:x86:*|cpe:2.3:a:fujitsu:interstage_application_server:12.0.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:12.0.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:12.1.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:12.1.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:12.2.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:12.2.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_information_integrator:11.3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_information_integrator:11.3.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_information_integrator_agent:11.3.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_security_control:1.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_security_control:1.0.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_security_control:1.0.0b:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_software_configuration_manager:15.6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_software_configuration_manager_express:15.6.0:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:datacenter:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:datacenter_without_hyper-v:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:enterprise:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:enterprise_without_hyper-v:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:foundation:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:standard:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:-:-:*:*:standard_without_hyper-v:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:datacenter:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:enterprise:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:foundation:*:x64:*|cpe:2.3:o:microsoft:windows_server_2008:r2:-:*:*:standard:*:x64:*|cpe:2.3:o:microsoft:windows_server_2012:-:*:*:*:datacenter:*:x64:*|cpe:2.3:o:microsoft:windows_server_2012:-:*:*:*:foundation:*:x64:*|cpe:2.3:o:microsoft:windows_server_2012:-:*:*:*:standard:*:x64:*|cpe:2.3:o:microsoft:windows_server_2016:-:*:*:*:datacenter:*:x64:*|cpe:2.3:o:microsoft:windows_server_2016:-:*:*:*:standard:*:x64:*|cpe:2.3:o:microsoft:windows_server_2019:-:*:*:*:datacenter:*:x64:*|cpe:2.3:o:microsoft:windows_server_2019:-:*:*:*:standard:*:x64:*|cpe:2.3:o:microsoft:windows_small_business_server_2011:-:*:*:*:essentials:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.2.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_development_cycle_manager:10.3.2:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.0b:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.1:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.1b:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.0.1b:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.2.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:9.2.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.1:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.1:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.3.1:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:10.0.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:10.0.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.0.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.0.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.1:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.1:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.1.1:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.2.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.2.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:interstage_application_server:11.2.0:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:11.2.0:*:*:*:standard-j:*:x64:*|cpe:2.3:a:fujitsu:interstage_list_works:10.4.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_web_server_express:11.1.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:linkexpress:5.0l20:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:linkexpress:5.0l21:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:safeauthor:3.6l10:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.1a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.1a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.9.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.9.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.9.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.9.1:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_software_configuration_manager:15.5.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_software_configuration_manager_express:15.5.0a:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:5.0:*:*:*:*:*:intel64:*|cpe:2.3:o:redhat:enterprise_linux:5.0:*:*:*:*:*:x86:*|cpe:2.3:o:redhat:enterprise_linux:6.0:*:*:*:*:*:intel64:*|cpe:2.3:o:redhat:enterprise_linux:6.0:*:*:*:*:*:x86:*|cpe:2.3:o:redhat:enterprise_linux:7.0:*:*:*:*:*:intel64:*|cpe:2.3:o:redhat:enterprise_linux:7.0:*:*:*:*:*:x86:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.2:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.2:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.1.0a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:9.1.0a:*:*:*:standard-j:*:*:*|cpe:2.3:a:fujitsu:interstage_job_workload_server:8.1.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:safeauthor:3.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:safeauthor:3.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:safeauthor:3.3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:safeauthor:3.4:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.0:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.4.1:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.6.0:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.6.1:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.7.0:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.7.0a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.7.0a:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.7.0a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0:*:*:*:global_enterprise:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0:*:*:*:standard:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0a:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0a:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0a:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0a:*:*:*:global_enterprise:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0a:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0a:*:*:*:standard:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0e:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:13.8.0e:*:*:*:standard:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0:*:*:*:enterprise:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0:*:*:*:global_enterprise:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.0:*:*:*:standard:*:x64:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.1:*:*:*:global_enterprise:*:*:*|cpe:2.3:a:fujitsu:systemwalker_operation_manager:16.0.1:*:*:*:standard:*:*:*|cpe:2.3:o:oracle:solaris:9:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2743,8 +3060,10 @@
       <c r="D68" t="n">
         <v>7.4</v>
       </c>
-      <c r="E68" t="n">
-        <v>3.1</v>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2756,8 +3075,11 @@
           <t>cpe:2.3:a:ntp:ntp:*:*:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:-:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta4:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-beta5:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-rc1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p1-rc2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p10:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p11:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p12:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p13:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2-rc1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2-rc2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p2-rc3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3-rc1:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3-rc2:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p3-rc3:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p4:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p5:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p6:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p7:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p8:*:*:*:*:*:*|cpe:2.3:a:ntp:ntp:4.2.8:p9:*:*:*:*:*:*|cpe:2.3:a:netapp:cloud_backup:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:clustered_data_ontap:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:data_ontap:-:*:*:*:*:7-mode:*:*|cpe:2.3:a:netapp:element_software:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:hci_management_node:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:ontap_tools:-:*:*:*:*:vmware_vsphere:*:*|cpe:2.3:a:netapp:solidfire:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:steelstore_cloud_integrated_storage:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:hci_compute_node_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:hci_compute_node:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h410c_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h410c:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h300s_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h300s:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h500s_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h500s:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h700s_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h700s:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h300e_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h300e:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h500e_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h500e:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h700e_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h700e:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:h410s_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:h410s:-:*:*:*:*:*:*:*|cpe:2.3:o:opensuse:leap:15.1:*:*:*:*:*:*:*|cpe:2.3:o:opensuse:leap:15.2:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2778,8 +3100,10 @@
       <c r="D69" t="n">
         <v>7.5</v>
       </c>
-      <c r="E69" t="n">
-        <v>3.1</v>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2791,8 +3115,11 @@
           <t>cpe:2.3:a:ise:smart_connect_knx_vaillant:1.2.839:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>vaillant</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2813,8 +3140,10 @@
       <c r="D70" t="n">
         <v>3.7</v>
       </c>
-      <c r="E70" t="n">
-        <v>3.1</v>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -2826,8 +3155,11 @@
           <t>cpe:2.3:a:openssl:openssl:*:*:*:*:*:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:16.04:*:*:*:lts:*:*:*|cpe:2.3:o:canonical:ubuntu_linux:18.04:*:*:*:lts:*:*:*|cpe:2.3:o:debian:debian_linux:9.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:jd_edwards_world_security:a9.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.56:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.57:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.58:*:*:*:*:*:*:*|cpe:2.3:o:oracle:ethernet_switch_es2-64_firmware:2.0.0.14:*:*:*:*:*:*:*|cpe:2.3:h:oracle:ethernet_switch_es2-64:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:ethernet_switch_es2-72_firmware:2.0.0.14:*:*:*:*:*:*:*|cpe:2.3:h:oracle:ethernet_switch_es2-72:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:ethernet_switch_es1-24_firmware:1.3.1:*:*:*:*:*:*:*|cpe:2.3:h:oracle:ethernet_switch_es1-24:-:*:*:*:*:*:*:*|cpe:2.3:o:oracle:ethernet_switch_tor-72_firmware:1.2.2:*:*:*:*:*:*:*|cpe:2.3:h:oracle:ethernet_switch_tor-72:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2848,8 +3180,10 @@
       <c r="D71" t="n">
         <v>7.8</v>
       </c>
-      <c r="E71" t="n">
-        <v>3.1</v>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2861,8 +3195,11 @@
           <t>cpe:2.3:a:haxx:curl:*:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:10.0:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinec_infrastructure_network_services:*:*:*:*:*:*:*:*|cpe:2.3:a:splunk:universal_forwarder:*:*:*:*:*:*:*:*|cpe:2.3:a:splunk:universal_forwarder:9.1.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2883,8 +3220,10 @@
       <c r="D72" t="n">
         <v>3.7</v>
       </c>
-      <c r="E72" t="n">
-        <v>3.1</v>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -2896,8 +3235,11 @@
           <t>cpe:2.3:a:haxx:curl:*:*:*:*:*:*:*:*|cpe:2.3:o:fedoraproject:fedora:32:*:*:*:*:*:*:*|cpe:2.3:o:fedoraproject:fedora:33:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:9.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:10.0:*:*:*:*:*:*:*|cpe:2.3:a:netapp:clustered_data_ontap:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:hci_management_node:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:solidfire:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:hci_storage_node:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:hci_bootstrap_os:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:hci_compute_node:-:*:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:*:*:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-002:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-004:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-005:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-006:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-007:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-002:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-003:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-004:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-005:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-006:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-007:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2021-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2021-002:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:supplemental_update:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:supplemental_update_2:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:-:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:security_update_2020:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:security_update_2020-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:security_update_2020-005:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:security_update_2020-007:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:security_update_2021-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:supplemental_update:*:*:*:*:*:*|cpe:2.3:o:apple:macos:11.0.1:*:*:*:*:*:*:*|cpe:2.3:o:apple:macos:11.1:*:*:*:*:*:*:*|cpe:2.3:o:apple:macos:11.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_billing_and_revenue_management:12.0.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_policy:1.14.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:essbase:21.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.58:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinec_infrastructure_network_services:*:*:*:*:*:*:*:*|cpe:2.3:a:splunk:universal_forwarder:*:*:*:*:*:*:*:*|cpe:2.3:a:splunk:universal_forwarder:9.1.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2918,8 +3260,10 @@
       <c r="D73" t="n">
         <v>7.5</v>
       </c>
-      <c r="E73" t="n">
-        <v>3.1</v>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -2931,8 +3275,11 @@
           <t>cpe:2.3:a:haxx:libcurl:*:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:9.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:10.0:*:*:*:*:*:*:*|cpe:2.3:o:fedoraproject:fedora:32:*:*:*:*:*:*:*|cpe:2.3:o:fedoraproject:fedora:33:*:*:*:*:*:*:*|cpe:2.3:a:netapp:clustered_data_ontap:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:hci_management_node:-:*:*:*:*:*:*:*|cpe:2.3:a:netapp:solidfire:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:hci_bootstrap_os:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:hci_compute_node:-:*:*:*:*:*:*:*|cpe:2.3:o:netapp:hci_storage_node_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:netapp:hci_storage_node:-:*:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:*:*:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:-:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2019-002:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-002:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-003:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-004:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-005:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-006:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2020-007:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.14.6:security_update_2021-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:-:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:security_update_2020-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:security_update_2021-001:*:*:*:*:*:*|cpe:2.3:o:apple:mac_os_x:10.15.7:supplemental_update:*:*:*:*:*:*|cpe:2.3:o:apple:macos:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_billing_and_revenue_management:12.0.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_policy:1.14.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:essbase:21.2:*:*:*:*:*:*:*|cpe:2.3:a:oracle:peoplesoft_enterprise_peopletools:8.58:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinec_infrastructure_network_services:*:*:*:*:*:*:*:*|cpe:2.3:a:splunk:universal_forwarder:*:*:*:*:*:*:*:*|cpe:2.3:a:splunk:universal_forwarder:9.1.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2953,8 +3300,10 @@
       <c r="D74" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E74" t="n">
-        <v>3.1</v>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -2966,8 +3315,11 @@
           <t>cpe:2.3:o:fujitsu:eternus_storage_dx200_s4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:eternus_storage_dx200_s4:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2988,8 +3340,10 @@
       <c r="D75" t="n">
         <v>7.5</v>
       </c>
-      <c r="E75" t="n">
-        <v>3.1</v>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -3001,8 +3355,11 @@
           <t>cpe:2.3:a:gnu:glibc:*:*:*:*:*:*:*:*|cpe:2.3:a:netapp:e-series_santricity_os_controller:*:*:*:*:*:*:*:*|cpe:2.3:a:netapp:ontap_select_deploy_administration_utility:-:*:*:*:*:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_security_edge_protection_proxy:1.5.0:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:10.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3023,8 +3380,10 @@
       <c r="D76" t="n">
         <v>7.8</v>
       </c>
-      <c r="E76" t="n">
-        <v>3.1</v>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3036,8 +3395,11 @@
           <t>cpe:2.3:a:fujitsu:scansnap_manager:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3058,8 +3420,10 @@
       <c r="D77" t="n">
         <v>7.5</v>
       </c>
-      <c r="E77" t="n">
-        <v>3.1</v>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3071,8 +3435,11 @@
           <t>cpe:2.3:a:openssl:openssl:*:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:10.0:*:*:*:*:*:*:*|cpe:2.3:a:tenable:log_correlation_engine:*:*:*:*:*:*:*:*|cpe:2.3:a:tenable:nessus_network_monitor:5.11.0:*:*:*:*:*:*:*|cpe:2.3:a:tenable:nessus_network_monitor:5.11.1:*:*:*:*:*:*:*|cpe:2.3:a:tenable:nessus_network_monitor:5.12.0:*:*:*:*:*:*:*|cpe:2.3:a:tenable:nessus_network_monitor:5.12.1:*:*:*:*:*:*:*|cpe:2.3:a:tenable:nessus_network_monitor:5.13.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:business_intelligence:5.5.0.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:business_intelligence:5.9.0.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:business_intelligence:12.2.1.3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:business_intelligence:12.2.1.4.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:communications_cloud_native_core_policy:1.15.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_manager_for_storage_management:13.4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:enterprise_manager_ops_center:12.4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:oracle:graalvm:19.3.5:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:graalvm:20.3.1.2:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:graalvm:21.0.0.2:*:*:*:enterprise:*:*:*|cpe:2.3:a:oracle:jd_edwards_enterpriseone_tools:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:jd_edwards_world_security:a9.4:*:*:*:*:*:*:*|cpe:2.3:a:oracle:mysql_server:*:*:*:*:*:*:*:*|cpe:2.3:a:oracle:nosql_database:*:*:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:*:*:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:-:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_1:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_10:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_2:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_3:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_4:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_5:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_6:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_7:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_8:*:*:*:*:*:*|cpe:2.3:a:mcafee:epolicy_orchestrator:5.10.0:update_9:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m10-4s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m10-4s:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:m12-2s_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:m12-2s:-:*:*:*:*:*:*:*|cpe:2.3:a:nodejs:node.js:*:*:*:*:-:*:*:*|cpe:2.3:a:nodejs:node.js:*:*:*:*:lts:*:*:*|cpe:2.3:a:nodejs:node.js:14.15.0:*:*:*:lts:*:*:*</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3093,8 +3460,10 @@
       <c r="D78" t="n">
         <v>5.4</v>
       </c>
-      <c r="E78" t="n">
-        <v>3.1</v>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -3106,8 +3475,11 @@
           <t>cpe:2.3:a:fujitsu:serverview_remote_management:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3128,8 +3500,10 @@
       <c r="D79" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E79" t="n">
-        <v>3.1</v>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3141,8 +3515,11 @@
           <t>cpe:2.3:o:fujitsu:ipcom_ex2_nw_1100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_nw_1100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_nw_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_nw_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_nw_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_nw_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_sc_1100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_sc_1100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_sc_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_sc_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_sc_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_sc_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_lb_1100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_lb_1100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_lb_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_lb_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_lb_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_lb_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_in_1100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_in_1100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_in_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_in_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_in_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_in_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_dc_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_dc_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_dc_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_dc_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_in_2300_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_in_2300:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_in_2500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_in_2500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_in_2700_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_in_2700:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_lb_1100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_lb_1100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_lb_1300_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_lb_1300:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_lb_2300_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_lb_2300:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_lb_2500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_lb_2500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_lb_2700_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_lb_2700:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_sc_1100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_sc_1100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_sc_1300_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_sc_1300:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_sc_2300_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_sc_2300:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_sc_2500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_sc_2500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_sc_2700_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_sc_2700:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_nw_1100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_nw_1100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_nw_1300_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_nw_1300:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_nw_2300_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_nw_2300:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_nw_2500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_nw_2500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex_nw_2700_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex_nw_2700:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus_100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus_100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus2_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus2_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus2_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus2_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_plus_100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_plus_100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_plus_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_plus_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_plus_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_plus_220:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3163,8 +3540,10 @@
       <c r="D80" t="n">
         <v>7.5</v>
       </c>
-      <c r="E80" t="n">
-        <v>3.1</v>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -3176,8 +3555,11 @@
           <t>cpe:2.3:o:fujitsu:ip-he950e_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-he950e:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-he950d_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-he950d:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-he900e_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-he900e:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-he900d_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-he900d:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-900e_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-900e:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-920e_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-920e:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-900d_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-900d:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-900iid_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-900iid:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-920d_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-920d:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-90_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-90:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ip-9610_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ip-9610:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3198,8 +3580,10 @@
       <c r="D81" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E81" t="n">
-        <v>3.1</v>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -3211,8 +3595,11 @@
           <t>cpe:2.3:o:fujitsu:si-r_30b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_30b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_130b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_130b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_90brin_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_90brin:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r570b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r570b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r370b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r370b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r220d_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r220d:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g100b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g100b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g110b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g110b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g200b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g200b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g210_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g210:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g211_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g211:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g120_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g120:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:si-r_g121_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:si-r_g121:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:sr-m_50ap1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:sr-m_50ap1:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3234,8 +3621,10 @@
       <c r="D82" t="n">
         <v>7.5</v>
       </c>
-      <c r="E82" t="n">
-        <v>3.1</v>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3247,8 +3636,11 @@
           <t>cpe:2.3:a:fujitsu:software_infrastructure_manager:2.8.0.060:*:*:*:advanced:-:*:*|cpe:2.3:a:fujitsu:software_infrastructure_manager:2.8.0.060:*:*:*:advanced:primeflex:*:*|cpe:2.3:a:fujitsu:software_infrastructure_manager:2.8.0.060:*:*:*:essential:*:*:*</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3269,8 +3661,10 @@
       <c r="D83" t="n">
         <v>5</v>
       </c>
-      <c r="E83" t="n">
-        <v>3.1</v>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3282,8 +3676,11 @@
           <t>cpe:2.3:a:fujitsu:software_infrastructure_manager:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3304,8 +3701,10 @@
       <c r="D84" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E84" t="n">
-        <v>3.1</v>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3317,8 +3716,11 @@
           <t>cpe:2.3:a:fujitsu:arconte_aurea:1.5.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3339,8 +3741,10 @@
       <c r="D85" t="n">
         <v>6.1</v>
       </c>
-      <c r="E85" t="n">
-        <v>3.1</v>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3352,8 +3756,11 @@
           <t>cpe:2.3:a:fujitsu:arconte_aurea:1.5.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3374,8 +3781,10 @@
       <c r="D86" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="E86" t="n">
-        <v>3.1</v>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -3387,8 +3796,11 @@
           <t>cpe:2.3:a:fujitsu:arconte_aurea:1.5.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3409,8 +3821,10 @@
       <c r="D87" t="n">
         <v>5.3</v>
       </c>
-      <c r="E87" t="n">
-        <v>3.1</v>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -3422,8 +3836,11 @@
           <t>cpe:2.3:a:fujitsu:arconte_aurea:1.5.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3444,8 +3861,10 @@
       <c r="D88" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="E88" t="n">
-        <v>3.1</v>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -3457,8 +3876,11 @@
           <t>cpe:2.3:a:fujitsu:arconte_aurea:1.5.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3479,8 +3901,10 @@
       <c r="D89" t="n">
         <v>5.5</v>
       </c>
-      <c r="E89" t="n">
-        <v>3.1</v>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -3492,8 +3916,11 @@
           <t>cpe:2.3:o:fujitsu:esprimo_d556\/2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d556\/2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d6011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d6011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d6012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d6012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d7010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d7010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d7010\/8_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d7010\/8:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d7011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d7011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d7012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d7012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d7013_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d7013:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d738_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d738:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d757_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d757:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d9010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d9010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d9011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d9011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d9012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d9012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d9013_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d9013:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d957_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d957:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d957\/e9x\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d957\/e9x\+:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_d958_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_d958:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_g5010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_g5010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_g5011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_g5011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_g558_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_g558:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_g6012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_g6012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_g9010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_g9010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_g9012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_g9012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_g9013_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_g9013:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_k5010\/24_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_k5010\/24:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_k557\/24_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_k557\/24:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_k558\/24_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_k558\/24:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p5010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p5010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p5011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p5011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p557_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p557:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p558\/power_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p558\/power:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p6012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p6012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p7010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p7010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p7011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p7011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p7012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p7012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p7013_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p7013:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p757_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p757:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p758_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p758:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p9010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p9010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p9011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p9011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p9012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p9012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p9013_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p9013:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p957_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p957:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9313x_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9313x:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u939_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u939:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u939x_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u939x:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9413_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9413:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:stylistic_q5010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:stylistic_q5010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:stylistic_q509_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:stylistic_q509:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:stylistic_q7310_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:stylistic_q7310:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:stylistic_q7311_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:stylistic_q7311:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:stylistic_q7312_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:stylistic_q7312:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:stylistic_q739_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:stylistic_q739:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primequest_3800b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primequest_3800b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primequest_3800b2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primequest_3800b2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primequest_3800e_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primequest_3800e:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primequest_3800e2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primequest_3800e2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primequest_4400e_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primequest_4400e:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_bx2560_m2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_bx2560_m2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_bx2580_m2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_bx2580_m2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2550_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2550_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2550_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2550_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2550_m6_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2550_m6:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2550_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2550_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2560_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2560_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2560_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2560_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2560_m6_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2560_m6:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2560_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2560_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2570_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2570_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_cx2570_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_cx2570_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_gx2460_m1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_gx2460_m1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_gx2560_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_gx2560_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_gx2570_m6_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_gx2570_m6:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx1330_m3_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx1330_m3:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx1330_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx1330_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx1330_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx1330_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx1440_m2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx1440_m2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2450_m1_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2450_m1:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2450_m2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2450_m2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2520_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2520_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2520_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2520_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2530_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2530_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2530_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2530_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p958_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p958:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p958\/power_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p958\/power:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_p9910_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_p9910:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q556\/2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q556\/2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q556\/2\/d_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q556\/2\/d:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q558_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q558:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q7010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q7010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q957\/mre_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q957\/:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q957_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q957:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q958_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q958:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:esprimo_q958\/mre_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:esprimo_q958\/mre:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_c780_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_c780:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_j5010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_j5010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_j550\/2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_j550\/2:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_j580_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_j580:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_m7010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_m7010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_m7010power_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_m7010power:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_m7010x_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_m7010x:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_m7010xpower_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_m7010xpower:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_r970_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_r970:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_r970b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_r970b:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_r970bpower_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_r970bpower:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w5010_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w5010:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w5010\/l_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w5010\/l:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w5011_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w5011:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w5012_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w5012:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w5012-ll_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w5012-ll:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w570_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w570:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w570power_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w570power:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w570power\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w570power\+:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w580_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w580:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w580power_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w580power:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_w580power\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_w580power\+:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_h5511_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_h5511:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_h7510_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_h7510:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_h7613_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_h7613:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_h780_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_h780:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:celsius_h980_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:celsius_h980:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_a3510_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_a3510:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_a3511_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_a3511:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2530_m6_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2530_m6:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2530_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2530_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2540_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2540_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2540_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2540_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2540_m6_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2540_m6:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx2540_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx2540_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx4770_m3_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx4770_m3:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx4770_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx4770_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx4770_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx4770_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx4770_m6_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx4770_m6:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx4770_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx4770_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_rx8770_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_rx8770_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1310_m3_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1310_m3:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1310_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1310_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1320_m3_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1320_m3:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1320_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1320_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1320_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1320_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1330_m3_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1330_m3:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1330_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1330_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx1330_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx1330_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx2550_m4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx2550_m4:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx2550_m5_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx2550_m5:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:primergy_tx2550_m7_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:primergy_tx2550_m7:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e4411_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e4411:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e4511_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e4511:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5410_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5410:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5411_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5411:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5412_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5412:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5412\/mtc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5412\/mtc:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5413_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5413:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e549_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e549:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5510_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5510:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5511_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5511:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5512_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5512:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e5513_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e5513:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e559_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e559:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e736_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e736:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e736_vpro_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e736_vpro:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e746_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e746:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_e746_vpro_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_e746_vpro:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_t939_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_t939:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u5313x_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u5313x:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u729_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u729:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u729x_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u729x:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7310_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7310:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7311_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7311:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7312_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7312:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7313_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7313:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7410_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7410:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7411_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7411:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7412_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7412:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7413_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7413:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u749_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u749:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7510_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7510:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7511_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7511:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7512_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7512:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u759_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u759:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u7613_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u7613:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9310_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9310:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9310x_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9310x:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9311_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9311:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9312_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9312:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:lifebook_u9312x_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:lifebook_u9312x:-:*:*:*:*:*:*:*|cpe:2.3:a:insyde:insydeh2o:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3518,8 +3945,10 @@
       <c r="D90" t="n">
         <v>5.5</v>
       </c>
-      <c r="E90" t="n">
-        <v>3.1</v>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -3531,8 +3960,11 @@
           <t>cpe:2.3:o:linux:linux_kernel:*:*:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:5.13:rc1:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:5.13:rc2:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3553,8 +3985,10 @@
       <c r="D91" t="n">
         <v>3.3</v>
       </c>
-      <c r="E91" t="n">
-        <v>3.1</v>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -3562,8 +3996,11 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3584,8 +4021,10 @@
       <c r="D92" t="n">
         <v>8.6</v>
       </c>
-      <c r="E92" t="n">
-        <v>3.1</v>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -3593,8 +4032,11 @@
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3615,8 +4057,10 @@
       <c r="D93" t="n">
         <v>6.5</v>
       </c>
-      <c r="E93" t="n">
-        <v>3.1</v>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -3624,8 +4068,11 @@
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3646,13 +4093,18 @@
       <c r="D94" t="n">
         <v>6.3</v>
       </c>
-      <c r="E94" t="n">
-        <v>3.1</v>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3673,8 +4125,10 @@
       <c r="D95" t="n">
         <v>7.5</v>
       </c>
-      <c r="E95" t="n">
-        <v>3.1</v>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -3686,8 +4140,11 @@
           <t>cpe:2.3:o:fujitsu:ipcom_ve2_ls_100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus_100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus_100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus2_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus2_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_ls_plus2_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_ls_plus2_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_plus_100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_plus_100:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_plus_200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_plus_200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ve2_sc_plus_220_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ve2_sc_plus_220:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_in_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_in_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_in_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_in_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_lb_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_lb_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_lb_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_lb_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_sc_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_sc_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_sc_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_sc_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_dc_3200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_dc_3200:-:*:*:*:*:*:*:*|cpe:2.3:o:fujitsu:ipcom_ex2_dc_3500_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fujitsu:ipcom_ex2_dc_3500:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3735,8 +4192,10 @@
       <c r="D96" t="n">
         <v>5.5</v>
       </c>
-      <c r="E96" t="n">
-        <v>3.1</v>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -3748,8 +4207,11 @@
           <t>cpe:2.3:o:linux:linux_kernel:*:*:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.13:rc1:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.13:rc2:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.13:rc3:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.13:rc4:*:*:*:*:*:*|cpe:2.3:o:linux:linux_kernel:6.13:rc5:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3770,8 +4232,10 @@
       <c r="D97" t="n">
         <v>6.5</v>
       </c>
-      <c r="E97" t="n">
-        <v>3.1</v>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -3779,8 +4243,11 @@
         </is>
       </c>
       <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>midea</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3801,13 +4268,18 @@
       <c r="D98" t="n">
         <v>7.5</v>
       </c>
-      <c r="E98" t="n">
-        <v>3.1</v>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>smartlife</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3828,8 +4300,10 @@
       <c r="D99" t="n">
         <v>7.5</v>
       </c>
-      <c r="E99" t="n">
-        <v>3.1</v>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -3837,8 +4311,11 @@
         </is>
       </c>
       <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
-      <c r="I99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>smartlife</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3859,8 +4336,10 @@
       <c r="D100" t="n">
         <v>7.7</v>
       </c>
-      <c r="E100" t="n">
-        <v>3.1</v>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -3872,8 +4351,11 @@
           <t>cpe:2.3:o:lsc:ptz_dual_band_camera_firmware:7.6.32:*:*:*:*:*:*:*|cpe:2.3:h:lsc:ptz_dual_band_camera:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3895,8 +4377,10 @@
       <c r="D101" t="n">
         <v>8</v>
       </c>
-      <c r="E101" t="n">
-        <v>3</v>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -3908,8 +4392,11 @@
           <t>cpe:2.3:o:wolfbox:level_2_ev_charger_firmware:3.1.17:*:*:*:*:*:*:*|cpe:2.3:h:wolfbox:level_2_ev_charger:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3931,8 +4418,10 @@
       <c r="D102" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E102" t="n">
-        <v>3</v>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -3944,8 +4433,11 @@
           <t>cpe:2.3:o:wolfbox:level_2_ev_charger_firmware:3.1.17:*:*:*:*:*:*:*|cpe:2.3:h:wolfbox:level_2_ev_charger:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3966,8 +4458,10 @@
       <c r="D103" t="n">
         <v>6.5</v>
       </c>
-      <c r="E103" t="n">
-        <v>3.1</v>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -3975,8 +4469,11 @@
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>air conditioner</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3997,8 +4494,10 @@
       <c r="D104" t="n">
         <v>9.1</v>
       </c>
-      <c r="E104" t="n">
-        <v>3.1</v>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -4010,8 +4509,11 @@
           <t>cpe:2.3:a:tuya:tuya:5.6.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4036,8 +4538,10 @@
       <c r="D105" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E105" t="n">
-        <v>3.1</v>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -4045,8 +4549,11 @@
         </is>
       </c>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>daikin</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4067,8 +4574,10 @@
       <c r="D106" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E106" t="n">
-        <v>3.1</v>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -4080,8 +4589,11 @@
           <t>cpe:2.3:a:tuya:smartlife:6.3.1:*:*:*:*:iphone_os:*:*|cpe:2.3:a:tuya:smartlife:6.3.4:*:*:*:*:android:*:*|cpe:2.3:a:tuya:tuya:*:*:*:*:*:android:*:*|cpe:2.3:a:tuya:tuya:*:*:*:*:*:iphone_os:*:*|cpe:2.3:a:tuya:tuya_smart:6.3.1:*:*:*:*:android:*:*|cpe:2.3:a:tuya:tuya_smart:6.3.1:*:*:*:*:iphone_os:*:*</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>smartlife|tuya</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4102,8 +4614,10 @@
       <c r="D107" t="n">
         <v>6.5</v>
       </c>
-      <c r="E107" t="n">
-        <v>3.1</v>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -4115,8 +4629,11 @@
           <t>cpe:2.3:o:keruistore:kerui_k259_firmware:33.53.87:*:*:*:*:*:*:*|cpe:2.3:h:keruistore:kerui_k259:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4137,8 +4654,10 @@
       <c r="D108" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="E108" t="n">
-        <v>3.1</v>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -4146,8 +4665,11 @@
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4168,8 +4690,10 @@
       <c r="D109" t="n">
         <v>7.5</v>
       </c>
-      <c r="E109" t="n">
-        <v>3.1</v>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -4177,8 +4701,11 @@
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4199,8 +4726,10 @@
       <c r="D110" t="n">
         <v>5.6</v>
       </c>
-      <c r="E110" t="n">
-        <v>3.1</v>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4208,8 +4737,11 @@
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4230,8 +4762,10 @@
       <c r="D111" t="n">
         <v>7.8</v>
       </c>
-      <c r="E111" t="n">
-        <v>3</v>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -4239,8 +4773,11 @@
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4261,8 +4798,10 @@
       <c r="D112" t="n">
         <v>3.1</v>
       </c>
-      <c r="E112" t="n">
-        <v>3.1</v>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -4270,8 +4809,11 @@
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4292,8 +4834,10 @@
       <c r="D113" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E113" t="n">
-        <v>3.1</v>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -4305,8 +4849,11 @@
           <t>cpe:2.3:a:tuya:arduino-tuyaopen:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4327,8 +4874,10 @@
       <c r="D114" t="n">
         <v>8.4</v>
       </c>
-      <c r="E114" t="n">
-        <v>3.1</v>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -4340,8 +4889,11 @@
           <t>cpe:2.3:a:tuya:arduino-tuyaopen:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4362,8 +4914,10 @@
       <c r="D115" t="n">
         <v>7.7</v>
       </c>
-      <c r="E115" t="n">
-        <v>3.1</v>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -4375,8 +4929,11 @@
           <t>cpe:2.3:a:tuya:arduino-tuyaopen:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4397,8 +4954,10 @@
       <c r="D116" t="n">
         <v>6.5</v>
       </c>
-      <c r="E116" t="n">
-        <v>3.1</v>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -4410,8 +4969,11 @@
           <t>cpe:2.3:a:tuya:arduino-tuyaopen:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>tuya</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4432,8 +4994,10 @@
       <c r="D117" t="n">
         <v>7.5</v>
       </c>
-      <c r="E117" t="n">
-        <v>3.1</v>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -4441,8 +5005,11 @@
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4468,8 +5035,11 @@
         </is>
       </c>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>air conditioner</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4490,8 +5060,10 @@
       <c r="D119" t="n">
         <v>4.3</v>
       </c>
-      <c r="E119" t="n">
-        <v>2</v>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
@@ -4499,8 +5071,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server:3.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:3.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:4.0:*:*:*:web_j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:*:*:web_j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:6.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:*:*:plus:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:*:*:standard:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:*:*:plus:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:*:*:standard_j:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.2:*:*:*:enterprise:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.2:*:*:*:standard_j:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks:6.0:*:*:ja:*:*:*:*</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4521,8 +5096,10 @@
       <c r="D120" t="n">
         <v>2.1</v>
       </c>
-      <c r="E120" t="n">
-        <v>2</v>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
@@ -4530,8 +5107,11 @@
           <t>cpe:2.3:a:fujitsu:fence:2:*:pro:*:*:*:*:*|cpe:2.3:a:fujitsu:fence:3:*:pro:*:*:*:*:*|cpe:2.3:a:fujitsu:fence:4:*:pro:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_encryption:v12.0l10:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_encryption:v12.0l10a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_encryption:v12.0l10b:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_encryption:v12.0l20:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:systemwalker_desktop_encryption:v13.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4552,8 +5132,10 @@
       <c r="D121" t="n">
         <v>5</v>
       </c>
-      <c r="E121" t="n">
-        <v>2</v>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -4565,8 +5147,11 @@
           <t>cpe:2.3:a:fujitsu:web_based_admin_view:2.1.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4587,8 +5172,10 @@
       <c r="D122" t="n">
         <v>6.4</v>
       </c>
-      <c r="E122" t="n">
-        <v>2</v>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
@@ -4596,8 +5183,11 @@
           <t>cpe:2.3:o:redhat:enterprise_linux:as_3:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:es_3:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v7.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:v7.0.0:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:as_4:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v7.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:v7.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.2:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:8.0.2:*:*:*:*:*:*:*|cpe:2.3:o:redhat:enterprise_linux:5.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:8.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v7.0:*:*:*:*:*:*:*|cpe:2.3:o:sun:solaris:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:7.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:9.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:7.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:9.0.0:*:*:*:*:*:*:*|cpe:2.3:o:microsoft:windows_nt:*:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_enterprise:v9.0.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:v6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus:v7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus_developer:v6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_plus_developer:v7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server_standard_j:v9.0.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_modelers_j:v6.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_modelers_j:v6.0a:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_apworks_modelers_j:v7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_enterprise:8.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_enterprise:v9.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_standard_j:8.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_studio_standard_j:v9.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_business_application_server_enterprise:v8.0.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4618,8 +5208,10 @@
       <c r="D123" t="n">
         <v>6.5</v>
       </c>
-      <c r="E123" t="n">
-        <v>2</v>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -4631,8 +5223,11 @@
           <t>cpe:2.3:a:fujitsu:serverview:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4653,8 +5248,10 @@
       <c r="D124" t="n">
         <v>5</v>
       </c>
-      <c r="E124" t="n">
-        <v>2</v>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
@@ -4662,8 +5259,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:standard:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:standard_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:web_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:web_j_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:enterprise_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus_developer:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus_developer_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:standard:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:enterprise_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:plus:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:plus_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:enterprise:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:enterprise_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:standard_j:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:standard_j_windows:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4684,8 +5284,10 @@
       <c r="D125" t="n">
         <v>5</v>
       </c>
-      <c r="E125" t="n">
-        <v>2</v>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -4693,8 +5295,11 @@
           <t>cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:standard_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:*:web_j_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:5.0:enterprise_windows:*:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:enterprise_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus_developer_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0:*:plus_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:enterprise_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:7.0.1:*:plus_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:enterprise_windows:*:*:*:*:*|cpe:2.3:a:fujitsu:interstage_application_server:8.0.0:*:standard_j_windows:*:*:*:*:*</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>fujitsu</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>